<commit_message>
Simple map: count stock in pallets only, drop units
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PaVB5ZWiX4HH2k96Bt3cJ6
</commit_message>
<xml_diff>
--- a/Floor_Map_Simple.xlsx
+++ b/Floor_Map_Simple.xlsx
@@ -474,20 +474,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblStock" displayName="tblStock" ref="A4:H6" headerRowCount="1">
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblStock" displayName="tblStock" ref="A4:F6" headerRowCount="1">
+  <tableColumns count="6">
     <tableColumn id="1" name="Item code"/>
     <tableColumn id="2" name="Description"/>
     <tableColumn id="3" name="Zone"/>
-    <tableColumn id="4" name="Units per pallet"/>
-    <tableColumn id="5" name="Low when pallets at or below"/>
-    <tableColumn id="6" name="Pallets on map">
+    <tableColumn id="4" name="Low when pallets at or below"/>
+    <tableColumn id="5" name="Pallets on map">
       <calculatedColumnFormula>IF(tblStock[[#This Row],[Item code]]="","",COUNTIF(Map!$A$6:$AJ$28,tblStock[[#This Row],[Item code]]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" name="Units on map">
-      <calculatedColumnFormula>IF(OR(tblStock[[#This Row],[Item code]]="",N(tblStock[[#This Row],[Units per pallet]])=0),"",tblStock[[#This Row],[Pallets on map]]*tblStock[[#This Row],[Units per pallet]])</calculatedColumnFormula>
-    </tableColumn>
-    <tableColumn id="8" name="Status">
+    <tableColumn id="6" name="Status">
       <calculatedColumnFormula>IF(tblStock[[#This Row],[Item code]]="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -893,7 +889,7 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Click a square  ▶  click the little arrow  ▶  pick the item.      To empty a square: click it and press Delete.</t>
+          <t>Click a square  →  click the little arrow  →  pick the item.      To empty a square: click it and press Delete.</t>
         </is>
       </c>
     </row>
@@ -1921,21 +1917,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1949,13 +1943,11 @@
       <c r="D1" s="2" t="n"/>
       <c r="E1" s="2" t="n"/>
       <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="26" t="inlineStr">
         <is>
-          <t>Type your items in the white columns. Grey columns fill in by themselves. Add a new item on the first empty row.</t>
+          <t>Everything is counted in PALLETS. Type your items in the white columns; grey columns fill in by themselves. Add a new item on the first empty row.</t>
         </is>
       </c>
     </row>
@@ -1977,45 +1969,35 @@
       </c>
       <c r="D4" s="27" t="inlineStr">
         <is>
-          <t>Units per pallet</t>
-        </is>
-      </c>
-      <c r="E4" s="27" t="inlineStr">
-        <is>
           <t>Low when pallets at or below</t>
         </is>
       </c>
+      <c r="E4" s="28" t="inlineStr">
+        <is>
+          <t>Pallets on map</t>
+        </is>
+      </c>
       <c r="F4" s="28" t="inlineStr">
         <is>
-          <t>Pallets on map</t>
-        </is>
-      </c>
-      <c r="G4" s="28" t="inlineStr">
-        <is>
-          <t>Units on map</t>
-        </is>
-      </c>
-      <c r="H4" s="28" t="inlineStr">
-        <is>
           <t>Status</t>
         </is>
       </c>
+      <c r="H4" s="29" t="inlineStr">
+        <is>
+          <t>Zone</t>
+        </is>
+      </c>
+      <c r="I4" s="29" t="inlineStr">
+        <is>
+          <t>Spaces</t>
+        </is>
+      </c>
       <c r="J4" s="29" t="inlineStr">
         <is>
-          <t>Zone</t>
+          <t>Used</t>
         </is>
       </c>
       <c r="K4" s="29" t="inlineStr">
-        <is>
-          <t>Spaces</t>
-        </is>
-      </c>
-      <c r="L4" s="29" t="inlineStr">
-        <is>
-          <t>Used</t>
-        </is>
-      </c>
-      <c r="M4" s="29" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
@@ -2037,36 +2019,29 @@
           <t>BOX</t>
         </is>
       </c>
-      <c r="D5" s="32" t="n">
-        <v>400</v>
-      </c>
-      <c r="E5" s="32" t="n"/>
-      <c r="F5" s="32">
+      <c r="D5" s="32" t="n"/>
+      <c r="E5" s="32">
         <f>IF(tblStock[[#This Row],[Item code]]="","",COUNTIF(Map!$A$6:$AJ$28,tblStock[[#This Row],[Item code]]))</f>
         <v/>
       </c>
-      <c r="G5" s="32">
-        <f>IF(OR(tblStock[[#This Row],[Item code]]="",N(tblStock[[#This Row],[Units per pallet]])=0),"",tblStock[[#This Row],[Pallets on map]]*tblStock[[#This Row],[Units per pallet]])</f>
-        <v/>
-      </c>
-      <c r="H5" s="30">
+      <c r="F5" s="30">
         <f>IF(tblStock[[#This Row],[Item code]]="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
         <v/>
       </c>
-      <c r="J5" s="33" t="inlineStr">
+      <c r="H5" s="33" t="inlineStr">
         <is>
           <t>Boxes</t>
         </is>
       </c>
-      <c r="K5" s="34" t="n">
+      <c r="I5" s="34" t="n">
         <v>256</v>
       </c>
-      <c r="L5" s="34">
+      <c r="J5" s="34">
         <f>COUNTA(Map!B18:Q21)+COUNTA(Map!B13:Q16)+COUNTA(Map!B8:Q11)+COUNTA(Map!U7:AJ10)</f>
         <v/>
       </c>
-      <c r="M5" s="35">
-        <f>K5-L5</f>
+      <c r="K5" s="35">
+        <f>I5-J5</f>
         <v/>
       </c>
     </row>
@@ -2086,86 +2061,79 @@
           <t>FLM</t>
         </is>
       </c>
-      <c r="D6" s="32" t="n">
-        <v>200</v>
-      </c>
-      <c r="E6" s="32" t="n"/>
-      <c r="F6" s="32">
+      <c r="D6" s="32" t="n"/>
+      <c r="E6" s="32">
         <f>IF(tblStock[[#This Row],[Item code]]="","",COUNTIF(Map!$A$6:$AJ$28,tblStock[[#This Row],[Item code]]))</f>
         <v/>
       </c>
-      <c r="G6" s="32">
-        <f>IF(OR(tblStock[[#This Row],[Item code]]="",N(tblStock[[#This Row],[Units per pallet]])=0),"",tblStock[[#This Row],[Pallets on map]]*tblStock[[#This Row],[Units per pallet]])</f>
-        <v/>
-      </c>
-      <c r="H6" s="30">
+      <c r="F6" s="30">
         <f>IF(tblStock[[#This Row],[Item code]]="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
         <v/>
       </c>
-      <c r="J6" s="36" t="inlineStr">
+      <c r="H6" s="36" t="inlineStr">
         <is>
           <t>Bags</t>
         </is>
       </c>
-      <c r="K6" s="34" t="n">
+      <c r="I6" s="34" t="n">
         <v>64</v>
       </c>
-      <c r="L6" s="34">
+      <c r="J6" s="34">
         <f>COUNTA(Map!U12:AJ15)</f>
         <v/>
       </c>
-      <c r="M6" s="35">
-        <f>K6-L6</f>
+      <c r="K6" s="35">
+        <f>I6-J6</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="J7" s="37" t="inlineStr">
+      <c r="H7" s="37" t="inlineStr">
         <is>
           <t>Films and Wrap</t>
         </is>
       </c>
-      <c r="K7" s="34" t="n">
+      <c r="I7" s="34" t="n">
         <v>64</v>
       </c>
-      <c r="L7" s="34">
+      <c r="J7" s="34">
         <f>COUNTA(Map!U17:AJ20)</f>
         <v/>
       </c>
-      <c r="M7" s="35">
-        <f>K7-L7</f>
+      <c r="K7" s="35">
+        <f>I7-J7</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="J8" s="38" t="inlineStr">
+      <c r="H8" s="38" t="inlineStr">
         <is>
           <t>Labels and Packing</t>
         </is>
       </c>
-      <c r="K8" s="34" t="n">
+      <c r="I8" s="34" t="n">
         <v>32</v>
       </c>
-      <c r="L8" s="34">
+      <c r="J8" s="34">
         <f>COUNTA(Map!U22:AJ23)</f>
         <v/>
       </c>
-      <c r="M8" s="35">
-        <f>K8-L8</f>
+      <c r="K8" s="35">
+        <f>I8-J8</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <conditionalFormatting sqref="H5:H304">
+  <conditionalFormatting sqref="F5:F304">
     <cfRule type="expression" priority="1" dxfId="5">
-      <formula>H5="LOW"</formula>
+      <formula>F5="LOW"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="6">
-      <formula>H5="OK"</formula>
+      <formula>F5="OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Simple map: zone names editable on the Stock sheet
Each zone name lives in one pink-bordered cell on Stock; aisle labels,
the map legend and free-space counts all read from it by formula.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PaVB5ZWiX4HH2k96Bt3cJ6
</commit_message>
<xml_diff>
--- a/Floor_Map_Simple.xlsx
+++ b/Floor_Map_Simple.xlsx
@@ -12,6 +12,10 @@
     <sheet name="Lists" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
+    <definedName name="zn_BOX">Stock!$I$5</definedName>
+    <definedName name="zn_BAG">Stock!$I$6</definedName>
+    <definedName name="zn_FLM">Stock!$I$7</definedName>
+    <definedName name="zn_LBL">Stock!$I$8</definedName>
     <definedName name="dd_ALL">OFFSET(Lists!$A$3,0,0,MAX(1,Lists!$A$2),1)</definedName>
     <definedName name="dd_BOX">OFFSET(Lists!$B$3,0,0,MAX(1,Lists!$B$2),1)</definedName>
     <definedName name="dd_BAG">OFFSET(Lists!$C$3,0,0,MAX(1,Lists!$C$2),1)</definedName>
@@ -28,7 +32,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,13 +75,18 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00E6007E"/>
+      <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="00E6007E"/>
       <sz val="12"/>
     </font>
     <font>
@@ -133,6 +142,30 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00C8A165"/>
+        <bgColor rgb="00C8A165"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004A90D9"/>
+        <bgColor rgb="004A90D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002BB3A3"/>
+        <bgColor rgb="002BB3A3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2B134"/>
+        <bgColor rgb="00F2B134"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="0000843D"/>
         <bgColor rgb="0000843D"/>
       </patternFill>
@@ -169,36 +202,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C8A165"/>
-        <bgColor rgb="00C8A165"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="004A90D9"/>
-        <bgColor rgb="004A90D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="002BB3A3"/>
-        <bgColor rgb="002BB3A3"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F2B134"/>
-        <bgColor rgb="00F2B134"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FF0000"/>
         <bgColor rgb="00FF0000"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -208,6 +217,20 @@
     </border>
     <border>
       <bottom style="thick">
+        <color rgb="00E6007E"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00E6007E"/>
+      </left>
+      <right style="medium">
+        <color rgb="00E6007E"/>
+      </right>
+      <top style="medium">
+        <color rgb="00E6007E"/>
+      </top>
+      <bottom style="medium">
         <color rgb="00E6007E"/>
       </bottom>
     </border>
@@ -229,63 +252,63 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -294,9 +317,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -307,16 +327,22 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -942,10 +968,9 @@
           <t>WALKWAY</t>
         </is>
       </c>
-      <c r="U6" s="7" t="inlineStr">
-        <is>
-          <t>R4   Boxes</t>
-        </is>
+      <c r="U6" s="7">
+        <f>"R4   "&amp;zn_BOX</f>
+        <v/>
       </c>
       <c r="AL6" s="8" t="inlineStr">
         <is>
@@ -963,10 +988,9 @@
       <c r="AU6" s="5" t="n"/>
     </row>
     <row r="7" ht="21" customHeight="1">
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>L3   Boxes</t>
-        </is>
+      <c r="B7" s="7">
+        <f>"L3   "&amp;zn_BOX</f>
+        <v/>
       </c>
       <c r="U7" s="9" t="n"/>
       <c r="V7" s="9" t="n"/>
@@ -985,10 +1009,9 @@
       <c r="AI7" s="9" t="n"/>
       <c r="AJ7" s="9" t="n"/>
       <c r="AL7" s="10" t="n"/>
-      <c r="AN7" s="11" t="inlineStr">
-        <is>
-          <t>Boxes</t>
-        </is>
+      <c r="AN7" s="11">
+        <f>zn_BOX</f>
+        <v/>
       </c>
     </row>
     <row r="8" ht="21" customHeight="1">
@@ -1025,10 +1048,9 @@
       <c r="AI8" s="9" t="n"/>
       <c r="AJ8" s="9" t="n"/>
       <c r="AL8" s="12" t="n"/>
-      <c r="AN8" s="11" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
+      <c r="AN8" s="11">
+        <f>zn_BAG</f>
+        <v/>
       </c>
     </row>
     <row r="9" ht="21" customHeight="1">
@@ -1065,10 +1087,9 @@
       <c r="AI9" s="9" t="n"/>
       <c r="AJ9" s="9" t="n"/>
       <c r="AL9" s="13" t="n"/>
-      <c r="AN9" s="11" t="inlineStr">
-        <is>
-          <t>Films and Wrap</t>
-        </is>
+      <c r="AN9" s="11">
+        <f>zn_FLM</f>
+        <v/>
       </c>
     </row>
     <row r="10" ht="21" customHeight="1">
@@ -1105,10 +1126,9 @@
       <c r="AI10" s="9" t="n"/>
       <c r="AJ10" s="9" t="n"/>
       <c r="AL10" s="14" t="n"/>
-      <c r="AN10" s="11" t="inlineStr">
-        <is>
-          <t>Labels and Packing</t>
-        </is>
+      <c r="AN10" s="11">
+        <f>zn_LBL</f>
+        <v/>
       </c>
     </row>
     <row r="11" ht="21" customHeight="1">
@@ -1128,10 +1148,9 @@
       <c r="O11" s="9" t="n"/>
       <c r="P11" s="9" t="n"/>
       <c r="Q11" s="9" t="n"/>
-      <c r="U11" s="7" t="inlineStr">
-        <is>
-          <t>R3   Bags</t>
-        </is>
+      <c r="U11" s="7">
+        <f>"R3   "&amp;zn_BAG</f>
+        <v/>
       </c>
       <c r="AL11" s="15" t="n"/>
       <c r="AN11" s="11" t="inlineStr">
@@ -1141,10 +1160,9 @@
       </c>
     </row>
     <row r="12" ht="21" customHeight="1">
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>L2   Boxes</t>
-        </is>
+      <c r="B12" s="7">
+        <f>"L2   "&amp;zn_BOX</f>
+        <v/>
       </c>
       <c r="U12" s="16" t="n"/>
       <c r="V12" s="16" t="n"/>
@@ -1308,26 +1326,23 @@
       <c r="O16" s="9" t="n"/>
       <c r="P16" s="9" t="n"/>
       <c r="Q16" s="9" t="n"/>
-      <c r="U16" s="7" t="inlineStr">
-        <is>
-          <t>R2   Films and Wrap</t>
-        </is>
+      <c r="U16" s="7">
+        <f>"R2   "&amp;zn_FLM</f>
+        <v/>
       </c>
       <c r="AL16" s="19">
         <f>256-(COUNTA(B18:Q21)+COUNTA(B13:Q16)+COUNTA(B8:Q11)+COUNTA(U7:AJ10))</f>
         <v/>
       </c>
-      <c r="AN16" s="11" t="inlineStr">
-        <is>
-          <t>Boxes</t>
-        </is>
+      <c r="AN16" s="11">
+        <f>zn_BOX</f>
+        <v/>
       </c>
     </row>
     <row r="17" ht="21" customHeight="1">
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>L1   Boxes</t>
-        </is>
+      <c r="B17" s="7">
+        <f>"L1   "&amp;zn_BOX</f>
+        <v/>
       </c>
       <c r="U17" s="20" t="n"/>
       <c r="V17" s="20" t="n"/>
@@ -1349,10 +1364,9 @@
         <f>64-(COUNTA(U12:AJ15))</f>
         <v/>
       </c>
-      <c r="AN17" s="11" t="inlineStr">
-        <is>
-          <t>Bags</t>
-        </is>
+      <c r="AN17" s="11">
+        <f>zn_BAG</f>
+        <v/>
       </c>
     </row>
     <row r="18" ht="21" customHeight="1">
@@ -1392,10 +1406,9 @@
         <f>64-(COUNTA(U17:AJ20))</f>
         <v/>
       </c>
-      <c r="AN18" s="11" t="inlineStr">
-        <is>
-          <t>Films and Wrap</t>
-        </is>
+      <c r="AN18" s="11">
+        <f>zn_FLM</f>
+        <v/>
       </c>
     </row>
     <row r="19" ht="21" customHeight="1">
@@ -1435,10 +1448,9 @@
         <f>32-(COUNTA(U22:AJ23))</f>
         <v/>
       </c>
-      <c r="AN19" s="11" t="inlineStr">
-        <is>
-          <t>Labels and Packing</t>
-        </is>
+      <c r="AN19" s="11">
+        <f>zn_LBL</f>
+        <v/>
       </c>
     </row>
     <row r="20" ht="21" customHeight="1">
@@ -1492,10 +1504,9 @@
       <c r="O21" s="9" t="n"/>
       <c r="P21" s="9" t="n"/>
       <c r="Q21" s="9" t="n"/>
-      <c r="U21" s="7" t="inlineStr">
-        <is>
-          <t>R1   Labels and Packing</t>
-        </is>
+      <c r="U21" s="7">
+        <f>"R1   "&amp;zn_LBL</f>
+        <v/>
       </c>
       <c r="AL21" s="8" t="inlineStr">
         <is>
@@ -1883,25 +1894,25 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="7">
-    <dataValidation sqref="B18:Q21" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not for this zone" error="That item isn't listed for this zone (or isn't on the Stock sheet). Put it here anyway?" promptTitle="L1  Boxes" prompt="Click the arrow and pick an item. Press Delete to empty." type="list" errorStyle="warning">
+    <dataValidation sqref="B18:Q21" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not for this zone" error="That item isn't listed for this zone (or isn't on the Stock sheet). Put it here anyway?" promptTitle="Aisle L1  (BOX)" prompt="Click the arrow and pick an item. Press Delete to empty." type="list" errorStyle="warning">
       <formula1>dd_BOX</formula1>
     </dataValidation>
-    <dataValidation sqref="B13:Q16" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not for this zone" error="That item isn't listed for this zone (or isn't on the Stock sheet). Put it here anyway?" promptTitle="L2  Boxes" prompt="Click the arrow and pick an item. Press Delete to empty." type="list" errorStyle="warning">
+    <dataValidation sqref="B13:Q16" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not for this zone" error="That item isn't listed for this zone (or isn't on the Stock sheet). Put it here anyway?" promptTitle="Aisle L2  (BOX)" prompt="Click the arrow and pick an item. Press Delete to empty." type="list" errorStyle="warning">
       <formula1>dd_BOX</formula1>
     </dataValidation>
-    <dataValidation sqref="B8:Q11" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not for this zone" error="That item isn't listed for this zone (or isn't on the Stock sheet). Put it here anyway?" promptTitle="L3  Boxes" prompt="Click the arrow and pick an item. Press Delete to empty." type="list" errorStyle="warning">
+    <dataValidation sqref="B8:Q11" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not for this zone" error="That item isn't listed for this zone (or isn't on the Stock sheet). Put it here anyway?" promptTitle="Aisle L3  (BOX)" prompt="Click the arrow and pick an item. Press Delete to empty." type="list" errorStyle="warning">
       <formula1>dd_BOX</formula1>
     </dataValidation>
-    <dataValidation sqref="U22:AJ23" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not for this zone" error="That item isn't listed for this zone (or isn't on the Stock sheet). Put it here anyway?" promptTitle="R1  Labels and Packing" prompt="Click the arrow and pick an item. Press Delete to empty." type="list" errorStyle="warning">
+    <dataValidation sqref="U22:AJ23" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not for this zone" error="That item isn't listed for this zone (or isn't on the Stock sheet). Put it here anyway?" promptTitle="Aisle R1  (LBL)" prompt="Click the arrow and pick an item. Press Delete to empty." type="list" errorStyle="warning">
       <formula1>dd_LBL</formula1>
     </dataValidation>
-    <dataValidation sqref="U17:AJ20" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not for this zone" error="That item isn't listed for this zone (or isn't on the Stock sheet). Put it here anyway?" promptTitle="R2  Films and Wrap" prompt="Click the arrow and pick an item. Press Delete to empty." type="list" errorStyle="warning">
+    <dataValidation sqref="U17:AJ20" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not for this zone" error="That item isn't listed for this zone (or isn't on the Stock sheet). Put it here anyway?" promptTitle="Aisle R2  (FLM)" prompt="Click the arrow and pick an item. Press Delete to empty." type="list" errorStyle="warning">
       <formula1>dd_FLM</formula1>
     </dataValidation>
-    <dataValidation sqref="U12:AJ15" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not for this zone" error="That item isn't listed for this zone (or isn't on the Stock sheet). Put it here anyway?" promptTitle="R3  Bags" prompt="Click the arrow and pick an item. Press Delete to empty." type="list" errorStyle="warning">
+    <dataValidation sqref="U12:AJ15" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not for this zone" error="That item isn't listed for this zone (or isn't on the Stock sheet). Put it here anyway?" promptTitle="Aisle R3  (BAG)" prompt="Click the arrow and pick an item. Press Delete to empty." type="list" errorStyle="warning">
       <formula1>dd_BAG</formula1>
     </dataValidation>
-    <dataValidation sqref="U7:AJ10" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not for this zone" error="That item isn't listed for this zone (or isn't on the Stock sheet). Put it here anyway?" promptTitle="R4  Boxes" prompt="Click the arrow and pick an item. Press Delete to empty." type="list" errorStyle="warning">
+    <dataValidation sqref="U7:AJ10" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Not for this zone" error="That item isn't listed for this zone (or isn't on the Stock sheet). Put it here anyway?" promptTitle="Aisle R4  (BOX)" prompt="Click the arrow and pick an item. Press Delete to empty." type="list" errorStyle="warning">
       <formula1>dd_BOX</formula1>
     </dataValidation>
   </dataValidations>
@@ -1917,7 +1928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1926,10 +1937,11 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1982,145 +1994,177 @@
           <t>Status</t>
         </is>
       </c>
-      <c r="H4" s="29" t="inlineStr">
+      <c r="H4" s="27" t="inlineStr">
         <is>
-          <t>Zone</t>
+          <t>Code</t>
         </is>
       </c>
-      <c r="I4" s="29" t="inlineStr">
+      <c r="I4" s="27" t="inlineStr">
+        <is>
+          <t>Zone name (you can change it)</t>
+        </is>
+      </c>
+      <c r="J4" s="27" t="inlineStr">
         <is>
           <t>Spaces</t>
         </is>
       </c>
-      <c r="J4" s="29" t="inlineStr">
+      <c r="K4" s="27" t="inlineStr">
         <is>
           <t>Used</t>
         </is>
       </c>
-      <c r="K4" s="29" t="inlineStr">
+      <c r="L4" s="27" t="inlineStr">
         <is>
           <t>Free</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>EX-BOX</t>
         </is>
       </c>
-      <c r="B5" s="31" t="inlineStr">
+      <c r="B5" s="30" t="inlineStr">
         <is>
           <t>EXAMPLE - type over me</t>
         </is>
       </c>
-      <c r="C5" s="32" t="inlineStr">
+      <c r="C5" s="31" t="inlineStr">
         <is>
           <t>BOX</t>
         </is>
       </c>
-      <c r="D5" s="32" t="n"/>
-      <c r="E5" s="32">
+      <c r="D5" s="31" t="n"/>
+      <c r="E5" s="31">
         <f>IF(tblStock[[#This Row],[Item code]]="","",COUNTIF(Map!$A$6:$AJ$28,tblStock[[#This Row],[Item code]]))</f>
         <v/>
       </c>
-      <c r="F5" s="30">
+      <c r="F5" s="29">
         <f>IF(tblStock[[#This Row],[Item code]]="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
         <v/>
       </c>
-      <c r="H5" s="33" t="inlineStr">
+      <c r="H5" s="32" t="inlineStr">
+        <is>
+          <t>BOX</t>
+        </is>
+      </c>
+      <c r="I5" s="33" t="inlineStr">
         <is>
           <t>Boxes</t>
         </is>
       </c>
-      <c r="I5" s="34" t="n">
+      <c r="J5" s="31" t="n">
         <v>256</v>
       </c>
-      <c r="J5" s="34">
+      <c r="K5" s="31">
         <f>COUNTA(Map!B18:Q21)+COUNTA(Map!B13:Q16)+COUNTA(Map!B8:Q11)+COUNTA(Map!U7:AJ10)</f>
         <v/>
       </c>
-      <c r="K5" s="35">
-        <f>I5-J5</f>
+      <c r="L5" s="29">
+        <f>J5-K5</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="30" t="inlineStr">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>EX-WRAP</t>
         </is>
       </c>
-      <c r="B6" s="31" t="inlineStr">
+      <c r="B6" s="30" t="inlineStr">
         <is>
           <t>EXAMPLE - type over me</t>
         </is>
       </c>
-      <c r="C6" s="32" t="inlineStr">
+      <c r="C6" s="31" t="inlineStr">
         <is>
           <t>FLM</t>
         </is>
       </c>
-      <c r="D6" s="32" t="n"/>
-      <c r="E6" s="32">
+      <c r="D6" s="31" t="n"/>
+      <c r="E6" s="31">
         <f>IF(tblStock[[#This Row],[Item code]]="","",COUNTIF(Map!$A$6:$AJ$28,tblStock[[#This Row],[Item code]]))</f>
         <v/>
       </c>
-      <c r="F6" s="30">
+      <c r="F6" s="29">
         <f>IF(tblStock[[#This Row],[Item code]]="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
         <v/>
       </c>
-      <c r="H6" s="36" t="inlineStr">
+      <c r="H6" s="34" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
+      </c>
+      <c r="I6" s="33" t="inlineStr">
         <is>
           <t>Bags</t>
         </is>
       </c>
-      <c r="I6" s="34" t="n">
+      <c r="J6" s="31" t="n">
         <v>64</v>
       </c>
-      <c r="J6" s="34">
+      <c r="K6" s="31">
         <f>COUNTA(Map!U12:AJ15)</f>
         <v/>
       </c>
-      <c r="K6" s="35">
-        <f>I6-J6</f>
+      <c r="L6" s="29">
+        <f>J6-K6</f>
         <v/>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="H7" s="37" t="inlineStr">
+      <c r="H7" s="35" t="inlineStr">
+        <is>
+          <t>FLM</t>
+        </is>
+      </c>
+      <c r="I7" s="33" t="inlineStr">
         <is>
           <t>Films and Wrap</t>
         </is>
       </c>
-      <c r="I7" s="34" t="n">
+      <c r="J7" s="31" t="n">
         <v>64</v>
       </c>
-      <c r="J7" s="34">
+      <c r="K7" s="31">
         <f>COUNTA(Map!U17:AJ20)</f>
         <v/>
       </c>
-      <c r="K7" s="35">
-        <f>I7-J7</f>
+      <c r="L7" s="29">
+        <f>J7-K7</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="H8" s="38" t="inlineStr">
+      <c r="H8" s="36" t="inlineStr">
+        <is>
+          <t>LBL</t>
+        </is>
+      </c>
+      <c r="I8" s="33" t="inlineStr">
         <is>
           <t>Labels and Packing</t>
         </is>
       </c>
-      <c r="I8" s="34" t="n">
+      <c r="J8" s="31" t="n">
         <v>32</v>
       </c>
-      <c r="J8" s="34">
+      <c r="K8" s="31">
         <f>COUNTA(Map!U22:AJ23)</f>
         <v/>
       </c>
-      <c r="K8" s="35">
-        <f>I8-J8</f>
-        <v/>
+      <c r="L8" s="29">
+        <f>J8-K8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="H9" s="37" t="inlineStr">
+        <is>
+          <t>Type over a zone name (pink box) and the Map changes too. In the Zone column on the left, use the Code.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Simple map: editable Layout sheet + Rebuild map macro
New Layout sheet (tblLayout) holds each aisle's side, order, rows,
pallets deep, zone and use. The Rebuild map button redraws the Map,
legend, Stock zone counts and the hidden Squares list from it, keeping
pallets by square name and logging any that no longer fit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PaVB5ZWiX4HH2k96Bt3cJ6
</commit_message>
<xml_diff>
--- a/Floor_Map_Simple.xlsx
+++ b/Floor_Map_Simple.xlsx
@@ -9,9 +9,10 @@
   <sheets>
     <sheet name="Map" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Stock" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Moves" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Lists" sheetId="4" state="hidden" r:id="rId4"/>
-    <sheet name="Squares" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet name="Layout" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Moves" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Lists" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet name="Squares" sheetId="6" state="hidden" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="zn_BOX">Stock!$I$5</definedName>
@@ -254,7 +255,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -345,6 +346,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -513,11 +515,27 @@
     <tableColumn id="3" name="Zone"/>
     <tableColumn id="4" name="Low when pallets at or below"/>
     <tableColumn id="5" name="Pallets on map">
-      <calculatedColumnFormula>IF(tblStock[[#This Row],[Item code]]="","",COUNTIF(Map!$A$6:$AJ$27,tblStock[[#This Row],[Item code]]))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(tblStock[[#This Row],[Item code]]="","",COUNTIF(Map!$A$6:$DZ$300,tblStock[[#This Row],[Item code]]))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" name="Status">
       <calculatedColumnFormula>IF(tblStock[[#This Row],[Item code]]="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</calculatedColumnFormula>
     </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium15" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblLayout" displayName="tblLayout" ref="A5:G14" headerRowCount="1">
+  <autoFilter ref="A5:G14"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="Aisle"/>
+    <tableColumn id="2" name="Side"/>
+    <tableColumn id="3" name="Order from fire exit"/>
+    <tableColumn id="4" name="Rows"/>
+    <tableColumn id="5" name="Pallets deep"/>
+    <tableColumn id="6" name="Zone"/>
+    <tableColumn id="7" name="Use"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showRowStripes="1"/>
 </table>
@@ -2026,7 +2044,7 @@
       </c>
       <c r="D5" s="31" t="n"/>
       <c r="E5" s="31">
-        <f>IF(tblStock[[#This Row],[Item code]]="","",COUNTIF(Map!$A$6:$AJ$27,tblStock[[#This Row],[Item code]]))</f>
+        <f>IF(tblStock[[#This Row],[Item code]]="","",COUNTIF(Map!$A$6:$DZ$300,tblStock[[#This Row],[Item code]]))</f>
         <v/>
       </c>
       <c r="F5" s="29">
@@ -2073,7 +2091,7 @@
       </c>
       <c r="D6" s="31" t="n"/>
       <c r="E6" s="31">
-        <f>IF(tblStock[[#This Row],[Item code]]="","",COUNTIF(Map!$A$6:$AJ$27,tblStock[[#This Row],[Item code]]))</f>
+        <f>IF(tblStock[[#This Row],[Item code]]="","",COUNTIF(Map!$A$6:$DZ$300,tblStock[[#This Row],[Item code]]))</f>
         <v/>
       </c>
       <c r="F6" s="29">
@@ -2187,6 +2205,422 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Layout</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="38" t="inlineStr">
+        <is>
+          <t>Change the numbers, then press the REBUILD MAP button. Pallets already on the map stay where they are.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>Aisle</t>
+        </is>
+      </c>
+      <c r="B5" s="27" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="C5" s="27" t="inlineStr">
+        <is>
+          <t>Order from fire exit</t>
+        </is>
+      </c>
+      <c r="D5" s="27" t="inlineStr">
+        <is>
+          <t>Rows</t>
+        </is>
+      </c>
+      <c r="E5" s="27" t="inlineStr">
+        <is>
+          <t>Pallets deep</t>
+        </is>
+      </c>
+      <c r="F5" s="27" t="inlineStr">
+        <is>
+          <t>Zone</t>
+        </is>
+      </c>
+      <c r="G5" s="27" t="inlineStr">
+        <is>
+          <t>Use</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="B6" s="31" t="inlineStr">
+        <is>
+          <t>Left</t>
+        </is>
+      </c>
+      <c r="C6" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="31" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" s="31" t="n">
+        <v>16</v>
+      </c>
+      <c r="F6" s="31" t="inlineStr"/>
+      <c r="G6" s="31" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>Left</t>
+        </is>
+      </c>
+      <c r="C7" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="31" t="n">
+        <v>4</v>
+      </c>
+      <c r="E7" s="31" t="n">
+        <v>16</v>
+      </c>
+      <c r="F7" s="31" t="inlineStr">
+        <is>
+          <t>BOX</t>
+        </is>
+      </c>
+      <c r="G7" s="31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="B8" s="31" t="inlineStr">
+        <is>
+          <t>Left</t>
+        </is>
+      </c>
+      <c r="C8" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" s="31" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" s="31" t="n">
+        <v>16</v>
+      </c>
+      <c r="F8" s="31" t="inlineStr">
+        <is>
+          <t>BOX</t>
+        </is>
+      </c>
+      <c r="G8" s="31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="29" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="B9" s="31" t="inlineStr">
+        <is>
+          <t>Left</t>
+        </is>
+      </c>
+      <c r="C9" s="31" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" s="31" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" s="31" t="n">
+        <v>16</v>
+      </c>
+      <c r="F9" s="31" t="inlineStr">
+        <is>
+          <t>BOX</t>
+        </is>
+      </c>
+      <c r="G9" s="31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="29" t="inlineStr">
+        <is>
+          <t>XR</t>
+        </is>
+      </c>
+      <c r="B10" s="31" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="C10" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="31" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" s="31" t="n">
+        <v>16</v>
+      </c>
+      <c r="F10" s="31" t="inlineStr"/>
+      <c r="G10" s="31" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="29" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B11" s="31" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="C11" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="31" t="n">
+        <v>16</v>
+      </c>
+      <c r="F11" s="31" t="inlineStr">
+        <is>
+          <t>LBL</t>
+        </is>
+      </c>
+      <c r="G11" s="31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="29" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B12" s="31" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="C12" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" s="31" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" s="31" t="n">
+        <v>16</v>
+      </c>
+      <c r="F12" s="31" t="inlineStr">
+        <is>
+          <t>FLM</t>
+        </is>
+      </c>
+      <c r="G12" s="31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="29" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="B13" s="31" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="C13" s="31" t="n">
+        <v>4</v>
+      </c>
+      <c r="D13" s="31" t="n">
+        <v>4</v>
+      </c>
+      <c r="E13" s="31" t="n">
+        <v>16</v>
+      </c>
+      <c r="F13" s="31" t="inlineStr">
+        <is>
+          <t>BAG</t>
+        </is>
+      </c>
+      <c r="G13" s="31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="29" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="B14" s="31" t="inlineStr">
+        <is>
+          <t>Right</t>
+        </is>
+      </c>
+      <c r="C14" s="31" t="n">
+        <v>5</v>
+      </c>
+      <c r="D14" s="31" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" s="31" t="n">
+        <v>16</v>
+      </c>
+      <c r="F14" s="31" t="inlineStr">
+        <is>
+          <t>BOX</t>
+        </is>
+      </c>
+      <c r="G14" s="31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="39" t="inlineStr">
+        <is>
+          <t>Rows = how many pallets wide the aisle is (1 row = 1 line of pallets on the map).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="39" t="inlineStr">
+        <is>
+          <t>Pallets deep = how many pallets from the walkway to the wall.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="39" t="inlineStr">
+        <is>
+          <t>Side: Left or Right, standing with the fire exit behind you. Order: 1 = nearest the fire exit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="39" t="inlineStr">
+        <is>
+          <t>Use: Yes = ours,  Blocked = someone else's (grey),  No = hide it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="39" t="inlineStr">
+        <is>
+          <t>Zone codes: BOX = Boxes,  BAG = Bags,  FLM = Films and Wrap,  LBL = Labels and Packing   (rename zones on the Stock sheet).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="39" t="inlineStr">
+        <is>
+          <t>New aisle? Type it on the first empty row under the table.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <dataValidations count="4">
+    <dataValidation sqref="B6:B60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Left,Right"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G6:G60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,Blocked,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F6:F60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"BOX,BAG,FLM,LBL"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C6:E60" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="Use a whole number from 1 to 60." type="whole" operator="between">
+      <formula1>1</formula1>
+      <formula2>60</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00808080"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2211,39 +2645,39 @@
       <c r="F1" s="2" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="38" t="inlineStr">
+      <c r="A2" s="39" t="inlineStr">
         <is>
           <t>Filled in automatically by the macros. Newest at the bottom.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="39" t="inlineStr">
+      <c r="A4" s="40" t="inlineStr">
         <is>
           <t>When</t>
         </is>
       </c>
-      <c r="B4" s="39" t="inlineStr">
+      <c r="B4" s="40" t="inlineStr">
         <is>
           <t>Who</t>
         </is>
       </c>
-      <c r="C4" s="39" t="inlineStr">
+      <c r="C4" s="40" t="inlineStr">
         <is>
           <t>What</t>
         </is>
       </c>
-      <c r="D4" s="39" t="inlineStr">
+      <c r="D4" s="40" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="E4" s="39" t="inlineStr">
+      <c r="E4" s="40" t="inlineStr">
         <is>
           <t>From</t>
         </is>
       </c>
-      <c r="F4" s="39" t="inlineStr">
+      <c r="F4" s="40" t="inlineStr">
         <is>
           <t>To</t>
         </is>
@@ -2257,7 +2691,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5620,7 +6054,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Fix Stock 'Pallets on map' count for new items
The Stock table now ships with 150 ready rows (formulas filled in), so
items typed on the next empty row count even when Excel doesn't grow
tables. Codes are trimmed before counting. Rebuild map now repairs the
Stock table in existing files (pulls in rows typed under it, rewrites
the count and status formulas) and the Map forces automatic calculation.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PaVB5ZWiX4HH2k96Bt3cJ6
</commit_message>
<xml_diff>
--- a/Floor_Map_Simple.xlsx
+++ b/Floor_Map_Simple.xlsx
@@ -508,17 +508,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblStock" displayName="tblStock" ref="A4:F6" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblStock" displayName="tblStock" ref="A4:F154" headerRowCount="1">
   <tableColumns count="6">
     <tableColumn id="1" name="Item code"/>
     <tableColumn id="2" name="Description"/>
     <tableColumn id="3" name="Zone"/>
     <tableColumn id="4" name="Low when pallets at or below"/>
     <tableColumn id="5" name="Pallets on map">
-      <calculatedColumnFormula>IF(tblStock[[#This Row],[Item code]]="","",COUNTIF(Map!$A$6:$DZ$300,tblStock[[#This Row],[Item code]]))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" name="Status">
-      <calculatedColumnFormula>IF(tblStock[[#This Row],[Item code]]="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showRowStripes="1"/>
@@ -1934,7 +1934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2044,11 +2044,11 @@
       </c>
       <c r="D5" s="31" t="n"/>
       <c r="E5" s="31">
-        <f>IF(tblStock[[#This Row],[Item code]]="","",COUNTIF(Map!$A$6:$DZ$300,tblStock[[#This Row],[Item code]]))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F5" s="29">
-        <f>IF(tblStock[[#This Row],[Item code]]="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
         <v/>
       </c>
       <c r="H5" s="32" t="inlineStr">
@@ -2091,11 +2091,11 @@
       </c>
       <c r="D6" s="31" t="n"/>
       <c r="E6" s="31">
-        <f>IF(tblStock[[#This Row],[Item code]]="","",COUNTIF(Map!$A$6:$DZ$300,tblStock[[#This Row],[Item code]]))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F6" s="29">
-        <f>IF(tblStock[[#This Row],[Item code]]="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
         <v/>
       </c>
       <c r="H6" s="34" t="inlineStr">
@@ -2121,6 +2121,18 @@
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="29" t="n"/>
+      <c r="B7" s="30" t="n"/>
+      <c r="C7" s="31" t="n"/>
+      <c r="D7" s="31" t="n"/>
+      <c r="E7" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F7" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
       <c r="H7" s="35" t="inlineStr">
         <is>
           <t>FLM</t>
@@ -2144,6 +2156,18 @@
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="29" t="n"/>
+      <c r="B8" s="30" t="n"/>
+      <c r="C8" s="31" t="n"/>
+      <c r="D8" s="31" t="n"/>
+      <c r="E8" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F8" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
       <c r="H8" s="36" t="inlineStr">
         <is>
           <t>LBL</t>
@@ -2166,11 +2190,2053 @@
         <v/>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="29" t="n"/>
+      <c r="B9" s="30" t="n"/>
+      <c r="C9" s="31" t="n"/>
+      <c r="D9" s="31" t="n"/>
+      <c r="E9" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F9" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
       <c r="H9" s="37" t="inlineStr">
         <is>
           <t>Type over a zone name (pink box) and the Map changes too. In the Zone column on the left, use the Code.</t>
         </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="29" t="n"/>
+      <c r="B10" s="30" t="n"/>
+      <c r="C10" s="31" t="n"/>
+      <c r="D10" s="31" t="n"/>
+      <c r="E10" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F10" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="29" t="n"/>
+      <c r="B11" s="30" t="n"/>
+      <c r="C11" s="31" t="n"/>
+      <c r="D11" s="31" t="n"/>
+      <c r="E11" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F11" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="29" t="n"/>
+      <c r="B12" s="30" t="n"/>
+      <c r="C12" s="31" t="n"/>
+      <c r="D12" s="31" t="n"/>
+      <c r="E12" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F12" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="29" t="n"/>
+      <c r="B13" s="30" t="n"/>
+      <c r="C13" s="31" t="n"/>
+      <c r="D13" s="31" t="n"/>
+      <c r="E13" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F13" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="29" t="n"/>
+      <c r="B14" s="30" t="n"/>
+      <c r="C14" s="31" t="n"/>
+      <c r="D14" s="31" t="n"/>
+      <c r="E14" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F14" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="29" t="n"/>
+      <c r="B15" s="30" t="n"/>
+      <c r="C15" s="31" t="n"/>
+      <c r="D15" s="31" t="n"/>
+      <c r="E15" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F15" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="29" t="n"/>
+      <c r="B16" s="30" t="n"/>
+      <c r="C16" s="31" t="n"/>
+      <c r="D16" s="31" t="n"/>
+      <c r="E16" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F16" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="29" t="n"/>
+      <c r="B17" s="30" t="n"/>
+      <c r="C17" s="31" t="n"/>
+      <c r="D17" s="31" t="n"/>
+      <c r="E17" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F17" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="29" t="n"/>
+      <c r="B18" s="30" t="n"/>
+      <c r="C18" s="31" t="n"/>
+      <c r="D18" s="31" t="n"/>
+      <c r="E18" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F18" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="29" t="n"/>
+      <c r="B19" s="30" t="n"/>
+      <c r="C19" s="31" t="n"/>
+      <c r="D19" s="31" t="n"/>
+      <c r="E19" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F19" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="29" t="n"/>
+      <c r="B20" s="30" t="n"/>
+      <c r="C20" s="31" t="n"/>
+      <c r="D20" s="31" t="n"/>
+      <c r="E20" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F20" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="29" t="n"/>
+      <c r="B21" s="30" t="n"/>
+      <c r="C21" s="31" t="n"/>
+      <c r="D21" s="31" t="n"/>
+      <c r="E21" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F21" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="29" t="n"/>
+      <c r="B22" s="30" t="n"/>
+      <c r="C22" s="31" t="n"/>
+      <c r="D22" s="31" t="n"/>
+      <c r="E22" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F22" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="29" t="n"/>
+      <c r="B23" s="30" t="n"/>
+      <c r="C23" s="31" t="n"/>
+      <c r="D23" s="31" t="n"/>
+      <c r="E23" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F23" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="29" t="n"/>
+      <c r="B24" s="30" t="n"/>
+      <c r="C24" s="31" t="n"/>
+      <c r="D24" s="31" t="n"/>
+      <c r="E24" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F24" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="29" t="n"/>
+      <c r="B25" s="30" t="n"/>
+      <c r="C25" s="31" t="n"/>
+      <c r="D25" s="31" t="n"/>
+      <c r="E25" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F25" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="29" t="n"/>
+      <c r="B26" s="30" t="n"/>
+      <c r="C26" s="31" t="n"/>
+      <c r="D26" s="31" t="n"/>
+      <c r="E26" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F26" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="29" t="n"/>
+      <c r="B27" s="30" t="n"/>
+      <c r="C27" s="31" t="n"/>
+      <c r="D27" s="31" t="n"/>
+      <c r="E27" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F27" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="29" t="n"/>
+      <c r="B28" s="30" t="n"/>
+      <c r="C28" s="31" t="n"/>
+      <c r="D28" s="31" t="n"/>
+      <c r="E28" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F28" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="29" t="n"/>
+      <c r="B29" s="30" t="n"/>
+      <c r="C29" s="31" t="n"/>
+      <c r="D29" s="31" t="n"/>
+      <c r="E29" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F29" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="29" t="n"/>
+      <c r="B30" s="30" t="n"/>
+      <c r="C30" s="31" t="n"/>
+      <c r="D30" s="31" t="n"/>
+      <c r="E30" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F30" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="29" t="n"/>
+      <c r="B31" s="30" t="n"/>
+      <c r="C31" s="31" t="n"/>
+      <c r="D31" s="31" t="n"/>
+      <c r="E31" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F31" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="29" t="n"/>
+      <c r="B32" s="30" t="n"/>
+      <c r="C32" s="31" t="n"/>
+      <c r="D32" s="31" t="n"/>
+      <c r="E32" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F32" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="29" t="n"/>
+      <c r="B33" s="30" t="n"/>
+      <c r="C33" s="31" t="n"/>
+      <c r="D33" s="31" t="n"/>
+      <c r="E33" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F33" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="29" t="n"/>
+      <c r="B34" s="30" t="n"/>
+      <c r="C34" s="31" t="n"/>
+      <c r="D34" s="31" t="n"/>
+      <c r="E34" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F34" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="29" t="n"/>
+      <c r="B35" s="30" t="n"/>
+      <c r="C35" s="31" t="n"/>
+      <c r="D35" s="31" t="n"/>
+      <c r="E35" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F35" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="29" t="n"/>
+      <c r="B36" s="30" t="n"/>
+      <c r="C36" s="31" t="n"/>
+      <c r="D36" s="31" t="n"/>
+      <c r="E36" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F36" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="29" t="n"/>
+      <c r="B37" s="30" t="n"/>
+      <c r="C37" s="31" t="n"/>
+      <c r="D37" s="31" t="n"/>
+      <c r="E37" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F37" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="29" t="n"/>
+      <c r="B38" s="30" t="n"/>
+      <c r="C38" s="31" t="n"/>
+      <c r="D38" s="31" t="n"/>
+      <c r="E38" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F38" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="29" t="n"/>
+      <c r="B39" s="30" t="n"/>
+      <c r="C39" s="31" t="n"/>
+      <c r="D39" s="31" t="n"/>
+      <c r="E39" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F39" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="29" t="n"/>
+      <c r="B40" s="30" t="n"/>
+      <c r="C40" s="31" t="n"/>
+      <c r="D40" s="31" t="n"/>
+      <c r="E40" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F40" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="29" t="n"/>
+      <c r="B41" s="30" t="n"/>
+      <c r="C41" s="31" t="n"/>
+      <c r="D41" s="31" t="n"/>
+      <c r="E41" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F41" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="29" t="n"/>
+      <c r="B42" s="30" t="n"/>
+      <c r="C42" s="31" t="n"/>
+      <c r="D42" s="31" t="n"/>
+      <c r="E42" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F42" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="29" t="n"/>
+      <c r="B43" s="30" t="n"/>
+      <c r="C43" s="31" t="n"/>
+      <c r="D43" s="31" t="n"/>
+      <c r="E43" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F43" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="29" t="n"/>
+      <c r="B44" s="30" t="n"/>
+      <c r="C44" s="31" t="n"/>
+      <c r="D44" s="31" t="n"/>
+      <c r="E44" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F44" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="29" t="n"/>
+      <c r="B45" s="30" t="n"/>
+      <c r="C45" s="31" t="n"/>
+      <c r="D45" s="31" t="n"/>
+      <c r="E45" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F45" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="29" t="n"/>
+      <c r="B46" s="30" t="n"/>
+      <c r="C46" s="31" t="n"/>
+      <c r="D46" s="31" t="n"/>
+      <c r="E46" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F46" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="29" t="n"/>
+      <c r="B47" s="30" t="n"/>
+      <c r="C47" s="31" t="n"/>
+      <c r="D47" s="31" t="n"/>
+      <c r="E47" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F47" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="29" t="n"/>
+      <c r="B48" s="30" t="n"/>
+      <c r="C48" s="31" t="n"/>
+      <c r="D48" s="31" t="n"/>
+      <c r="E48" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F48" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="29" t="n"/>
+      <c r="B49" s="30" t="n"/>
+      <c r="C49" s="31" t="n"/>
+      <c r="D49" s="31" t="n"/>
+      <c r="E49" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F49" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="29" t="n"/>
+      <c r="B50" s="30" t="n"/>
+      <c r="C50" s="31" t="n"/>
+      <c r="D50" s="31" t="n"/>
+      <c r="E50" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F50" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="29" t="n"/>
+      <c r="B51" s="30" t="n"/>
+      <c r="C51" s="31" t="n"/>
+      <c r="D51" s="31" t="n"/>
+      <c r="E51" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F51" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="29" t="n"/>
+      <c r="B52" s="30" t="n"/>
+      <c r="C52" s="31" t="n"/>
+      <c r="D52" s="31" t="n"/>
+      <c r="E52" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F52" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="29" t="n"/>
+      <c r="B53" s="30" t="n"/>
+      <c r="C53" s="31" t="n"/>
+      <c r="D53" s="31" t="n"/>
+      <c r="E53" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F53" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="29" t="n"/>
+      <c r="B54" s="30" t="n"/>
+      <c r="C54" s="31" t="n"/>
+      <c r="D54" s="31" t="n"/>
+      <c r="E54" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F54" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="29" t="n"/>
+      <c r="B55" s="30" t="n"/>
+      <c r="C55" s="31" t="n"/>
+      <c r="D55" s="31" t="n"/>
+      <c r="E55" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F55" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="29" t="n"/>
+      <c r="B56" s="30" t="n"/>
+      <c r="C56" s="31" t="n"/>
+      <c r="D56" s="31" t="n"/>
+      <c r="E56" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F56" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="29" t="n"/>
+      <c r="B57" s="30" t="n"/>
+      <c r="C57" s="31" t="n"/>
+      <c r="D57" s="31" t="n"/>
+      <c r="E57" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F57" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="29" t="n"/>
+      <c r="B58" s="30" t="n"/>
+      <c r="C58" s="31" t="n"/>
+      <c r="D58" s="31" t="n"/>
+      <c r="E58" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F58" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="29" t="n"/>
+      <c r="B59" s="30" t="n"/>
+      <c r="C59" s="31" t="n"/>
+      <c r="D59" s="31" t="n"/>
+      <c r="E59" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F59" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="29" t="n"/>
+      <c r="B60" s="30" t="n"/>
+      <c r="C60" s="31" t="n"/>
+      <c r="D60" s="31" t="n"/>
+      <c r="E60" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F60" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="29" t="n"/>
+      <c r="B61" s="30" t="n"/>
+      <c r="C61" s="31" t="n"/>
+      <c r="D61" s="31" t="n"/>
+      <c r="E61" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F61" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="29" t="n"/>
+      <c r="B62" s="30" t="n"/>
+      <c r="C62" s="31" t="n"/>
+      <c r="D62" s="31" t="n"/>
+      <c r="E62" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F62" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="29" t="n"/>
+      <c r="B63" s="30" t="n"/>
+      <c r="C63" s="31" t="n"/>
+      <c r="D63" s="31" t="n"/>
+      <c r="E63" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F63" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64" ht="22" customHeight="1">
+      <c r="A64" s="29" t="n"/>
+      <c r="B64" s="30" t="n"/>
+      <c r="C64" s="31" t="n"/>
+      <c r="D64" s="31" t="n"/>
+      <c r="E64" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F64" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65" ht="22" customHeight="1">
+      <c r="A65" s="29" t="n"/>
+      <c r="B65" s="30" t="n"/>
+      <c r="C65" s="31" t="n"/>
+      <c r="D65" s="31" t="n"/>
+      <c r="E65" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F65" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66" ht="22" customHeight="1">
+      <c r="A66" s="29" t="n"/>
+      <c r="B66" s="30" t="n"/>
+      <c r="C66" s="31" t="n"/>
+      <c r="D66" s="31" t="n"/>
+      <c r="E66" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F66" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="29" t="n"/>
+      <c r="B67" s="30" t="n"/>
+      <c r="C67" s="31" t="n"/>
+      <c r="D67" s="31" t="n"/>
+      <c r="E67" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F67" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68" ht="22" customHeight="1">
+      <c r="A68" s="29" t="n"/>
+      <c r="B68" s="30" t="n"/>
+      <c r="C68" s="31" t="n"/>
+      <c r="D68" s="31" t="n"/>
+      <c r="E68" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F68" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69" ht="22" customHeight="1">
+      <c r="A69" s="29" t="n"/>
+      <c r="B69" s="30" t="n"/>
+      <c r="C69" s="31" t="n"/>
+      <c r="D69" s="31" t="n"/>
+      <c r="E69" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F69" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="29" t="n"/>
+      <c r="B70" s="30" t="n"/>
+      <c r="C70" s="31" t="n"/>
+      <c r="D70" s="31" t="n"/>
+      <c r="E70" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F70" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71" ht="22" customHeight="1">
+      <c r="A71" s="29" t="n"/>
+      <c r="B71" s="30" t="n"/>
+      <c r="C71" s="31" t="n"/>
+      <c r="D71" s="31" t="n"/>
+      <c r="E71" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F71" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72" ht="22" customHeight="1">
+      <c r="A72" s="29" t="n"/>
+      <c r="B72" s="30" t="n"/>
+      <c r="C72" s="31" t="n"/>
+      <c r="D72" s="31" t="n"/>
+      <c r="E72" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F72" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" ht="22" customHeight="1">
+      <c r="A73" s="29" t="n"/>
+      <c r="B73" s="30" t="n"/>
+      <c r="C73" s="31" t="n"/>
+      <c r="D73" s="31" t="n"/>
+      <c r="E73" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F73" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="29" t="n"/>
+      <c r="B74" s="30" t="n"/>
+      <c r="C74" s="31" t="n"/>
+      <c r="D74" s="31" t="n"/>
+      <c r="E74" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F74" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75" ht="22" customHeight="1">
+      <c r="A75" s="29" t="n"/>
+      <c r="B75" s="30" t="n"/>
+      <c r="C75" s="31" t="n"/>
+      <c r="D75" s="31" t="n"/>
+      <c r="E75" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F75" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76" ht="22" customHeight="1">
+      <c r="A76" s="29" t="n"/>
+      <c r="B76" s="30" t="n"/>
+      <c r="C76" s="31" t="n"/>
+      <c r="D76" s="31" t="n"/>
+      <c r="E76" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F76" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" s="29" t="n"/>
+      <c r="B77" s="30" t="n"/>
+      <c r="C77" s="31" t="n"/>
+      <c r="D77" s="31" t="n"/>
+      <c r="E77" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F77" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="29" t="n"/>
+      <c r="B78" s="30" t="n"/>
+      <c r="C78" s="31" t="n"/>
+      <c r="D78" s="31" t="n"/>
+      <c r="E78" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F78" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79" ht="22" customHeight="1">
+      <c r="A79" s="29" t="n"/>
+      <c r="B79" s="30" t="n"/>
+      <c r="C79" s="31" t="n"/>
+      <c r="D79" s="31" t="n"/>
+      <c r="E79" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F79" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80" ht="22" customHeight="1">
+      <c r="A80" s="29" t="n"/>
+      <c r="B80" s="30" t="n"/>
+      <c r="C80" s="31" t="n"/>
+      <c r="D80" s="31" t="n"/>
+      <c r="E80" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F80" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81" ht="22" customHeight="1">
+      <c r="A81" s="29" t="n"/>
+      <c r="B81" s="30" t="n"/>
+      <c r="C81" s="31" t="n"/>
+      <c r="D81" s="31" t="n"/>
+      <c r="E81" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F81" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82" ht="22" customHeight="1">
+      <c r="A82" s="29" t="n"/>
+      <c r="B82" s="30" t="n"/>
+      <c r="C82" s="31" t="n"/>
+      <c r="D82" s="31" t="n"/>
+      <c r="E82" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F82" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83" ht="22" customHeight="1">
+      <c r="A83" s="29" t="n"/>
+      <c r="B83" s="30" t="n"/>
+      <c r="C83" s="31" t="n"/>
+      <c r="D83" s="31" t="n"/>
+      <c r="E83" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F83" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84" ht="22" customHeight="1">
+      <c r="A84" s="29" t="n"/>
+      <c r="B84" s="30" t="n"/>
+      <c r="C84" s="31" t="n"/>
+      <c r="D84" s="31" t="n"/>
+      <c r="E84" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F84" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85" ht="22" customHeight="1">
+      <c r="A85" s="29" t="n"/>
+      <c r="B85" s="30" t="n"/>
+      <c r="C85" s="31" t="n"/>
+      <c r="D85" s="31" t="n"/>
+      <c r="E85" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F85" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86" ht="22" customHeight="1">
+      <c r="A86" s="29" t="n"/>
+      <c r="B86" s="30" t="n"/>
+      <c r="C86" s="31" t="n"/>
+      <c r="D86" s="31" t="n"/>
+      <c r="E86" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F86" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87" ht="22" customHeight="1">
+      <c r="A87" s="29" t="n"/>
+      <c r="B87" s="30" t="n"/>
+      <c r="C87" s="31" t="n"/>
+      <c r="D87" s="31" t="n"/>
+      <c r="E87" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F87" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88" ht="22" customHeight="1">
+      <c r="A88" s="29" t="n"/>
+      <c r="B88" s="30" t="n"/>
+      <c r="C88" s="31" t="n"/>
+      <c r="D88" s="31" t="n"/>
+      <c r="E88" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F88" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89" ht="22" customHeight="1">
+      <c r="A89" s="29" t="n"/>
+      <c r="B89" s="30" t="n"/>
+      <c r="C89" s="31" t="n"/>
+      <c r="D89" s="31" t="n"/>
+      <c r="E89" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F89" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90" ht="22" customHeight="1">
+      <c r="A90" s="29" t="n"/>
+      <c r="B90" s="30" t="n"/>
+      <c r="C90" s="31" t="n"/>
+      <c r="D90" s="31" t="n"/>
+      <c r="E90" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F90" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91" ht="22" customHeight="1">
+      <c r="A91" s="29" t="n"/>
+      <c r="B91" s="30" t="n"/>
+      <c r="C91" s="31" t="n"/>
+      <c r="D91" s="31" t="n"/>
+      <c r="E91" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F91" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92" ht="22" customHeight="1">
+      <c r="A92" s="29" t="n"/>
+      <c r="B92" s="30" t="n"/>
+      <c r="C92" s="31" t="n"/>
+      <c r="D92" s="31" t="n"/>
+      <c r="E92" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F92" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93" ht="22" customHeight="1">
+      <c r="A93" s="29" t="n"/>
+      <c r="B93" s="30" t="n"/>
+      <c r="C93" s="31" t="n"/>
+      <c r="D93" s="31" t="n"/>
+      <c r="E93" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F93" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94" ht="22" customHeight="1">
+      <c r="A94" s="29" t="n"/>
+      <c r="B94" s="30" t="n"/>
+      <c r="C94" s="31" t="n"/>
+      <c r="D94" s="31" t="n"/>
+      <c r="E94" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F94" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95" ht="22" customHeight="1">
+      <c r="A95" s="29" t="n"/>
+      <c r="B95" s="30" t="n"/>
+      <c r="C95" s="31" t="n"/>
+      <c r="D95" s="31" t="n"/>
+      <c r="E95" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F95" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96" ht="22" customHeight="1">
+      <c r="A96" s="29" t="n"/>
+      <c r="B96" s="30" t="n"/>
+      <c r="C96" s="31" t="n"/>
+      <c r="D96" s="31" t="n"/>
+      <c r="E96" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F96" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97" ht="22" customHeight="1">
+      <c r="A97" s="29" t="n"/>
+      <c r="B97" s="30" t="n"/>
+      <c r="C97" s="31" t="n"/>
+      <c r="D97" s="31" t="n"/>
+      <c r="E97" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F97" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98" ht="22" customHeight="1">
+      <c r="A98" s="29" t="n"/>
+      <c r="B98" s="30" t="n"/>
+      <c r="C98" s="31" t="n"/>
+      <c r="D98" s="31" t="n"/>
+      <c r="E98" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F98" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99" ht="22" customHeight="1">
+      <c r="A99" s="29" t="n"/>
+      <c r="B99" s="30" t="n"/>
+      <c r="C99" s="31" t="n"/>
+      <c r="D99" s="31" t="n"/>
+      <c r="E99" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F99" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100" ht="22" customHeight="1">
+      <c r="A100" s="29" t="n"/>
+      <c r="B100" s="30" t="n"/>
+      <c r="C100" s="31" t="n"/>
+      <c r="D100" s="31" t="n"/>
+      <c r="E100" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F100" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101" ht="22" customHeight="1">
+      <c r="A101" s="29" t="n"/>
+      <c r="B101" s="30" t="n"/>
+      <c r="C101" s="31" t="n"/>
+      <c r="D101" s="31" t="n"/>
+      <c r="E101" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F101" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102" ht="22" customHeight="1">
+      <c r="A102" s="29" t="n"/>
+      <c r="B102" s="30" t="n"/>
+      <c r="C102" s="31" t="n"/>
+      <c r="D102" s="31" t="n"/>
+      <c r="E102" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F102" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103" ht="22" customHeight="1">
+      <c r="A103" s="29" t="n"/>
+      <c r="B103" s="30" t="n"/>
+      <c r="C103" s="31" t="n"/>
+      <c r="D103" s="31" t="n"/>
+      <c r="E103" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F103" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104" ht="22" customHeight="1">
+      <c r="A104" s="29" t="n"/>
+      <c r="B104" s="30" t="n"/>
+      <c r="C104" s="31" t="n"/>
+      <c r="D104" s="31" t="n"/>
+      <c r="E104" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F104" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="105" ht="22" customHeight="1">
+      <c r="A105" s="29" t="n"/>
+      <c r="B105" s="30" t="n"/>
+      <c r="C105" s="31" t="n"/>
+      <c r="D105" s="31" t="n"/>
+      <c r="E105" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F105" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="106" ht="22" customHeight="1">
+      <c r="A106" s="29" t="n"/>
+      <c r="B106" s="30" t="n"/>
+      <c r="C106" s="31" t="n"/>
+      <c r="D106" s="31" t="n"/>
+      <c r="E106" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F106" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="107" ht="22" customHeight="1">
+      <c r="A107" s="29" t="n"/>
+      <c r="B107" s="30" t="n"/>
+      <c r="C107" s="31" t="n"/>
+      <c r="D107" s="31" t="n"/>
+      <c r="E107" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F107" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="108" ht="22" customHeight="1">
+      <c r="A108" s="29" t="n"/>
+      <c r="B108" s="30" t="n"/>
+      <c r="C108" s="31" t="n"/>
+      <c r="D108" s="31" t="n"/>
+      <c r="E108" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F108" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="109" ht="22" customHeight="1">
+      <c r="A109" s="29" t="n"/>
+      <c r="B109" s="30" t="n"/>
+      <c r="C109" s="31" t="n"/>
+      <c r="D109" s="31" t="n"/>
+      <c r="E109" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F109" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="110" ht="22" customHeight="1">
+      <c r="A110" s="29" t="n"/>
+      <c r="B110" s="30" t="n"/>
+      <c r="C110" s="31" t="n"/>
+      <c r="D110" s="31" t="n"/>
+      <c r="E110" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F110" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="111" ht="22" customHeight="1">
+      <c r="A111" s="29" t="n"/>
+      <c r="B111" s="30" t="n"/>
+      <c r="C111" s="31" t="n"/>
+      <c r="D111" s="31" t="n"/>
+      <c r="E111" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F111" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112" ht="22" customHeight="1">
+      <c r="A112" s="29" t="n"/>
+      <c r="B112" s="30" t="n"/>
+      <c r="C112" s="31" t="n"/>
+      <c r="D112" s="31" t="n"/>
+      <c r="E112" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F112" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113" ht="22" customHeight="1">
+      <c r="A113" s="29" t="n"/>
+      <c r="B113" s="30" t="n"/>
+      <c r="C113" s="31" t="n"/>
+      <c r="D113" s="31" t="n"/>
+      <c r="E113" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F113" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114" ht="22" customHeight="1">
+      <c r="A114" s="29" t="n"/>
+      <c r="B114" s="30" t="n"/>
+      <c r="C114" s="31" t="n"/>
+      <c r="D114" s="31" t="n"/>
+      <c r="E114" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F114" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="115" ht="22" customHeight="1">
+      <c r="A115" s="29" t="n"/>
+      <c r="B115" s="30" t="n"/>
+      <c r="C115" s="31" t="n"/>
+      <c r="D115" s="31" t="n"/>
+      <c r="E115" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F115" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="116" ht="22" customHeight="1">
+      <c r="A116" s="29" t="n"/>
+      <c r="B116" s="30" t="n"/>
+      <c r="C116" s="31" t="n"/>
+      <c r="D116" s="31" t="n"/>
+      <c r="E116" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F116" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="117" ht="22" customHeight="1">
+      <c r="A117" s="29" t="n"/>
+      <c r="B117" s="30" t="n"/>
+      <c r="C117" s="31" t="n"/>
+      <c r="D117" s="31" t="n"/>
+      <c r="E117" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F117" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="118" ht="22" customHeight="1">
+      <c r="A118" s="29" t="n"/>
+      <c r="B118" s="30" t="n"/>
+      <c r="C118" s="31" t="n"/>
+      <c r="D118" s="31" t="n"/>
+      <c r="E118" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F118" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="119" ht="22" customHeight="1">
+      <c r="A119" s="29" t="n"/>
+      <c r="B119" s="30" t="n"/>
+      <c r="C119" s="31" t="n"/>
+      <c r="D119" s="31" t="n"/>
+      <c r="E119" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F119" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="120" ht="22" customHeight="1">
+      <c r="A120" s="29" t="n"/>
+      <c r="B120" s="30" t="n"/>
+      <c r="C120" s="31" t="n"/>
+      <c r="D120" s="31" t="n"/>
+      <c r="E120" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F120" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121" ht="22" customHeight="1">
+      <c r="A121" s="29" t="n"/>
+      <c r="B121" s="30" t="n"/>
+      <c r="C121" s="31" t="n"/>
+      <c r="D121" s="31" t="n"/>
+      <c r="E121" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F121" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="122" ht="22" customHeight="1">
+      <c r="A122" s="29" t="n"/>
+      <c r="B122" s="30" t="n"/>
+      <c r="C122" s="31" t="n"/>
+      <c r="D122" s="31" t="n"/>
+      <c r="E122" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F122" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="123" ht="22" customHeight="1">
+      <c r="A123" s="29" t="n"/>
+      <c r="B123" s="30" t="n"/>
+      <c r="C123" s="31" t="n"/>
+      <c r="D123" s="31" t="n"/>
+      <c r="E123" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F123" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="124" ht="22" customHeight="1">
+      <c r="A124" s="29" t="n"/>
+      <c r="B124" s="30" t="n"/>
+      <c r="C124" s="31" t="n"/>
+      <c r="D124" s="31" t="n"/>
+      <c r="E124" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F124" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="125" ht="22" customHeight="1">
+      <c r="A125" s="29" t="n"/>
+      <c r="B125" s="30" t="n"/>
+      <c r="C125" s="31" t="n"/>
+      <c r="D125" s="31" t="n"/>
+      <c r="E125" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F125" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="126" ht="22" customHeight="1">
+      <c r="A126" s="29" t="n"/>
+      <c r="B126" s="30" t="n"/>
+      <c r="C126" s="31" t="n"/>
+      <c r="D126" s="31" t="n"/>
+      <c r="E126" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F126" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="127" ht="22" customHeight="1">
+      <c r="A127" s="29" t="n"/>
+      <c r="B127" s="30" t="n"/>
+      <c r="C127" s="31" t="n"/>
+      <c r="D127" s="31" t="n"/>
+      <c r="E127" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F127" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="128" ht="22" customHeight="1">
+      <c r="A128" s="29" t="n"/>
+      <c r="B128" s="30" t="n"/>
+      <c r="C128" s="31" t="n"/>
+      <c r="D128" s="31" t="n"/>
+      <c r="E128" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F128" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="129" ht="22" customHeight="1">
+      <c r="A129" s="29" t="n"/>
+      <c r="B129" s="30" t="n"/>
+      <c r="C129" s="31" t="n"/>
+      <c r="D129" s="31" t="n"/>
+      <c r="E129" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F129" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="130" ht="22" customHeight="1">
+      <c r="A130" s="29" t="n"/>
+      <c r="B130" s="30" t="n"/>
+      <c r="C130" s="31" t="n"/>
+      <c r="D130" s="31" t="n"/>
+      <c r="E130" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F130" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="131" ht="22" customHeight="1">
+      <c r="A131" s="29" t="n"/>
+      <c r="B131" s="30" t="n"/>
+      <c r="C131" s="31" t="n"/>
+      <c r="D131" s="31" t="n"/>
+      <c r="E131" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F131" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="132" ht="22" customHeight="1">
+      <c r="A132" s="29" t="n"/>
+      <c r="B132" s="30" t="n"/>
+      <c r="C132" s="31" t="n"/>
+      <c r="D132" s="31" t="n"/>
+      <c r="E132" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F132" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="133" ht="22" customHeight="1">
+      <c r="A133" s="29" t="n"/>
+      <c r="B133" s="30" t="n"/>
+      <c r="C133" s="31" t="n"/>
+      <c r="D133" s="31" t="n"/>
+      <c r="E133" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F133" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="134" ht="22" customHeight="1">
+      <c r="A134" s="29" t="n"/>
+      <c r="B134" s="30" t="n"/>
+      <c r="C134" s="31" t="n"/>
+      <c r="D134" s="31" t="n"/>
+      <c r="E134" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F134" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="135" ht="22" customHeight="1">
+      <c r="A135" s="29" t="n"/>
+      <c r="B135" s="30" t="n"/>
+      <c r="C135" s="31" t="n"/>
+      <c r="D135" s="31" t="n"/>
+      <c r="E135" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F135" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="136" ht="22" customHeight="1">
+      <c r="A136" s="29" t="n"/>
+      <c r="B136" s="30" t="n"/>
+      <c r="C136" s="31" t="n"/>
+      <c r="D136" s="31" t="n"/>
+      <c r="E136" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F136" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="137" ht="22" customHeight="1">
+      <c r="A137" s="29" t="n"/>
+      <c r="B137" s="30" t="n"/>
+      <c r="C137" s="31" t="n"/>
+      <c r="D137" s="31" t="n"/>
+      <c r="E137" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F137" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="138" ht="22" customHeight="1">
+      <c r="A138" s="29" t="n"/>
+      <c r="B138" s="30" t="n"/>
+      <c r="C138" s="31" t="n"/>
+      <c r="D138" s="31" t="n"/>
+      <c r="E138" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F138" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="139" ht="22" customHeight="1">
+      <c r="A139" s="29" t="n"/>
+      <c r="B139" s="30" t="n"/>
+      <c r="C139" s="31" t="n"/>
+      <c r="D139" s="31" t="n"/>
+      <c r="E139" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F139" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="140" ht="22" customHeight="1">
+      <c r="A140" s="29" t="n"/>
+      <c r="B140" s="30" t="n"/>
+      <c r="C140" s="31" t="n"/>
+      <c r="D140" s="31" t="n"/>
+      <c r="E140" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F140" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="141" ht="22" customHeight="1">
+      <c r="A141" s="29" t="n"/>
+      <c r="B141" s="30" t="n"/>
+      <c r="C141" s="31" t="n"/>
+      <c r="D141" s="31" t="n"/>
+      <c r="E141" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F141" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="142" ht="22" customHeight="1">
+      <c r="A142" s="29" t="n"/>
+      <c r="B142" s="30" t="n"/>
+      <c r="C142" s="31" t="n"/>
+      <c r="D142" s="31" t="n"/>
+      <c r="E142" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F142" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="143" ht="22" customHeight="1">
+      <c r="A143" s="29" t="n"/>
+      <c r="B143" s="30" t="n"/>
+      <c r="C143" s="31" t="n"/>
+      <c r="D143" s="31" t="n"/>
+      <c r="E143" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F143" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="144" ht="22" customHeight="1">
+      <c r="A144" s="29" t="n"/>
+      <c r="B144" s="30" t="n"/>
+      <c r="C144" s="31" t="n"/>
+      <c r="D144" s="31" t="n"/>
+      <c r="E144" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F144" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="145" ht="22" customHeight="1">
+      <c r="A145" s="29" t="n"/>
+      <c r="B145" s="30" t="n"/>
+      <c r="C145" s="31" t="n"/>
+      <c r="D145" s="31" t="n"/>
+      <c r="E145" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F145" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="146" ht="22" customHeight="1">
+      <c r="A146" s="29" t="n"/>
+      <c r="B146" s="30" t="n"/>
+      <c r="C146" s="31" t="n"/>
+      <c r="D146" s="31" t="n"/>
+      <c r="E146" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F146" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="147" ht="22" customHeight="1">
+      <c r="A147" s="29" t="n"/>
+      <c r="B147" s="30" t="n"/>
+      <c r="C147" s="31" t="n"/>
+      <c r="D147" s="31" t="n"/>
+      <c r="E147" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F147" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="148" ht="22" customHeight="1">
+      <c r="A148" s="29" t="n"/>
+      <c r="B148" s="30" t="n"/>
+      <c r="C148" s="31" t="n"/>
+      <c r="D148" s="31" t="n"/>
+      <c r="E148" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F148" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="149" ht="22" customHeight="1">
+      <c r="A149" s="29" t="n"/>
+      <c r="B149" s="30" t="n"/>
+      <c r="C149" s="31" t="n"/>
+      <c r="D149" s="31" t="n"/>
+      <c r="E149" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F149" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="150" ht="22" customHeight="1">
+      <c r="A150" s="29" t="n"/>
+      <c r="B150" s="30" t="n"/>
+      <c r="C150" s="31" t="n"/>
+      <c r="D150" s="31" t="n"/>
+      <c r="E150" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F150" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="151" ht="22" customHeight="1">
+      <c r="A151" s="29" t="n"/>
+      <c r="B151" s="30" t="n"/>
+      <c r="C151" s="31" t="n"/>
+      <c r="D151" s="31" t="n"/>
+      <c r="E151" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F151" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="152" ht="22" customHeight="1">
+      <c r="A152" s="29" t="n"/>
+      <c r="B152" s="30" t="n"/>
+      <c r="C152" s="31" t="n"/>
+      <c r="D152" s="31" t="n"/>
+      <c r="E152" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F152" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="153" ht="22" customHeight="1">
+      <c r="A153" s="29" t="n"/>
+      <c r="B153" s="30" t="n"/>
+      <c r="C153" s="31" t="n"/>
+      <c r="D153" s="31" t="n"/>
+      <c r="E153" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F153" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="154" ht="22" customHeight="1">
+      <c r="A154" s="29" t="n"/>
+      <c r="B154" s="30" t="n"/>
+      <c r="C154" s="31" t="n"/>
+      <c r="D154" s="31" t="n"/>
+      <c r="E154" s="31">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <v/>
+      </c>
+      <c r="F154" s="29">
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Stock count covers the whole Map and self-repairs
'Pallets on map' counted only up to a fixed column, so pallets in wider
maps showed 0. Count over Map!A6:ZZ2000, and have the macros check the
formula on first use and rewrite it if it is old or was edited.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PaVB5ZWiX4HH2k96Bt3cJ6
</commit_message>
<xml_diff>
--- a/Floor_Map_Simple.xlsx
+++ b/Floor_Map_Simple.xlsx
@@ -515,7 +515,7 @@
     <tableColumn id="3" name="Zone"/>
     <tableColumn id="4" name="Low when pallets at or below"/>
     <tableColumn id="5" name="Pallets on map">
-      <calculatedColumnFormula>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" name="Status">
       <calculatedColumnFormula>IF(TRIM(tblStock[[#This Row],[Item code]])="","",IF(tblStock[[#This Row],[Pallets on map]]&lt;=IF(tblStock[[#This Row],[Low when pallets at or below]]="",2,tblStock[[#This Row],[Low when pallets at or below]]),"LOW","OK"))</calculatedColumnFormula>
@@ -2044,7 +2044,7 @@
       </c>
       <c r="D5" s="31" t="n"/>
       <c r="E5" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F5" s="29">
@@ -2091,7 +2091,7 @@
       </c>
       <c r="D6" s="31" t="n"/>
       <c r="E6" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F6" s="29">
@@ -2126,7 +2126,7 @@
       <c r="C7" s="31" t="n"/>
       <c r="D7" s="31" t="n"/>
       <c r="E7" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F7" s="29">
@@ -2161,7 +2161,7 @@
       <c r="C8" s="31" t="n"/>
       <c r="D8" s="31" t="n"/>
       <c r="E8" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F8" s="29">
@@ -2196,7 +2196,7 @@
       <c r="C9" s="31" t="n"/>
       <c r="D9" s="31" t="n"/>
       <c r="E9" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F9" s="29">
@@ -2215,7 +2215,7 @@
       <c r="C10" s="31" t="n"/>
       <c r="D10" s="31" t="n"/>
       <c r="E10" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F10" s="29">
@@ -2229,7 +2229,7 @@
       <c r="C11" s="31" t="n"/>
       <c r="D11" s="31" t="n"/>
       <c r="E11" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F11" s="29">
@@ -2243,7 +2243,7 @@
       <c r="C12" s="31" t="n"/>
       <c r="D12" s="31" t="n"/>
       <c r="E12" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F12" s="29">
@@ -2257,7 +2257,7 @@
       <c r="C13" s="31" t="n"/>
       <c r="D13" s="31" t="n"/>
       <c r="E13" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F13" s="29">
@@ -2271,7 +2271,7 @@
       <c r="C14" s="31" t="n"/>
       <c r="D14" s="31" t="n"/>
       <c r="E14" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F14" s="29">
@@ -2285,7 +2285,7 @@
       <c r="C15" s="31" t="n"/>
       <c r="D15" s="31" t="n"/>
       <c r="E15" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F15" s="29">
@@ -2299,7 +2299,7 @@
       <c r="C16" s="31" t="n"/>
       <c r="D16" s="31" t="n"/>
       <c r="E16" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F16" s="29">
@@ -2313,7 +2313,7 @@
       <c r="C17" s="31" t="n"/>
       <c r="D17" s="31" t="n"/>
       <c r="E17" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F17" s="29">
@@ -2327,7 +2327,7 @@
       <c r="C18" s="31" t="n"/>
       <c r="D18" s="31" t="n"/>
       <c r="E18" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F18" s="29">
@@ -2341,7 +2341,7 @@
       <c r="C19" s="31" t="n"/>
       <c r="D19" s="31" t="n"/>
       <c r="E19" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F19" s="29">
@@ -2355,7 +2355,7 @@
       <c r="C20" s="31" t="n"/>
       <c r="D20" s="31" t="n"/>
       <c r="E20" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F20" s="29">
@@ -2369,7 +2369,7 @@
       <c r="C21" s="31" t="n"/>
       <c r="D21" s="31" t="n"/>
       <c r="E21" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F21" s="29">
@@ -2383,7 +2383,7 @@
       <c r="C22" s="31" t="n"/>
       <c r="D22" s="31" t="n"/>
       <c r="E22" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F22" s="29">
@@ -2397,7 +2397,7 @@
       <c r="C23" s="31" t="n"/>
       <c r="D23" s="31" t="n"/>
       <c r="E23" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F23" s="29">
@@ -2411,7 +2411,7 @@
       <c r="C24" s="31" t="n"/>
       <c r="D24" s="31" t="n"/>
       <c r="E24" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F24" s="29">
@@ -2425,7 +2425,7 @@
       <c r="C25" s="31" t="n"/>
       <c r="D25" s="31" t="n"/>
       <c r="E25" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F25" s="29">
@@ -2439,7 +2439,7 @@
       <c r="C26" s="31" t="n"/>
       <c r="D26" s="31" t="n"/>
       <c r="E26" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F26" s="29">
@@ -2453,7 +2453,7 @@
       <c r="C27" s="31" t="n"/>
       <c r="D27" s="31" t="n"/>
       <c r="E27" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F27" s="29">
@@ -2467,7 +2467,7 @@
       <c r="C28" s="31" t="n"/>
       <c r="D28" s="31" t="n"/>
       <c r="E28" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F28" s="29">
@@ -2481,7 +2481,7 @@
       <c r="C29" s="31" t="n"/>
       <c r="D29" s="31" t="n"/>
       <c r="E29" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F29" s="29">
@@ -2495,7 +2495,7 @@
       <c r="C30" s="31" t="n"/>
       <c r="D30" s="31" t="n"/>
       <c r="E30" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F30" s="29">
@@ -2509,7 +2509,7 @@
       <c r="C31" s="31" t="n"/>
       <c r="D31" s="31" t="n"/>
       <c r="E31" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F31" s="29">
@@ -2523,7 +2523,7 @@
       <c r="C32" s="31" t="n"/>
       <c r="D32" s="31" t="n"/>
       <c r="E32" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F32" s="29">
@@ -2537,7 +2537,7 @@
       <c r="C33" s="31" t="n"/>
       <c r="D33" s="31" t="n"/>
       <c r="E33" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F33" s="29">
@@ -2551,7 +2551,7 @@
       <c r="C34" s="31" t="n"/>
       <c r="D34" s="31" t="n"/>
       <c r="E34" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F34" s="29">
@@ -2565,7 +2565,7 @@
       <c r="C35" s="31" t="n"/>
       <c r="D35" s="31" t="n"/>
       <c r="E35" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F35" s="29">
@@ -2579,7 +2579,7 @@
       <c r="C36" s="31" t="n"/>
       <c r="D36" s="31" t="n"/>
       <c r="E36" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F36" s="29">
@@ -2593,7 +2593,7 @@
       <c r="C37" s="31" t="n"/>
       <c r="D37" s="31" t="n"/>
       <c r="E37" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F37" s="29">
@@ -2607,7 +2607,7 @@
       <c r="C38" s="31" t="n"/>
       <c r="D38" s="31" t="n"/>
       <c r="E38" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F38" s="29">
@@ -2621,7 +2621,7 @@
       <c r="C39" s="31" t="n"/>
       <c r="D39" s="31" t="n"/>
       <c r="E39" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F39" s="29">
@@ -2635,7 +2635,7 @@
       <c r="C40" s="31" t="n"/>
       <c r="D40" s="31" t="n"/>
       <c r="E40" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F40" s="29">
@@ -2649,7 +2649,7 @@
       <c r="C41" s="31" t="n"/>
       <c r="D41" s="31" t="n"/>
       <c r="E41" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F41" s="29">
@@ -2663,7 +2663,7 @@
       <c r="C42" s="31" t="n"/>
       <c r="D42" s="31" t="n"/>
       <c r="E42" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F42" s="29">
@@ -2677,7 +2677,7 @@
       <c r="C43" s="31" t="n"/>
       <c r="D43" s="31" t="n"/>
       <c r="E43" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F43" s="29">
@@ -2691,7 +2691,7 @@
       <c r="C44" s="31" t="n"/>
       <c r="D44" s="31" t="n"/>
       <c r="E44" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F44" s="29">
@@ -2705,7 +2705,7 @@
       <c r="C45" s="31" t="n"/>
       <c r="D45" s="31" t="n"/>
       <c r="E45" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F45" s="29">
@@ -2719,7 +2719,7 @@
       <c r="C46" s="31" t="n"/>
       <c r="D46" s="31" t="n"/>
       <c r="E46" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F46" s="29">
@@ -2733,7 +2733,7 @@
       <c r="C47" s="31" t="n"/>
       <c r="D47" s="31" t="n"/>
       <c r="E47" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F47" s="29">
@@ -2747,7 +2747,7 @@
       <c r="C48" s="31" t="n"/>
       <c r="D48" s="31" t="n"/>
       <c r="E48" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F48" s="29">
@@ -2761,7 +2761,7 @@
       <c r="C49" s="31" t="n"/>
       <c r="D49" s="31" t="n"/>
       <c r="E49" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F49" s="29">
@@ -2775,7 +2775,7 @@
       <c r="C50" s="31" t="n"/>
       <c r="D50" s="31" t="n"/>
       <c r="E50" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F50" s="29">
@@ -2789,7 +2789,7 @@
       <c r="C51" s="31" t="n"/>
       <c r="D51" s="31" t="n"/>
       <c r="E51" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F51" s="29">
@@ -2803,7 +2803,7 @@
       <c r="C52" s="31" t="n"/>
       <c r="D52" s="31" t="n"/>
       <c r="E52" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F52" s="29">
@@ -2817,7 +2817,7 @@
       <c r="C53" s="31" t="n"/>
       <c r="D53" s="31" t="n"/>
       <c r="E53" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F53" s="29">
@@ -2831,7 +2831,7 @@
       <c r="C54" s="31" t="n"/>
       <c r="D54" s="31" t="n"/>
       <c r="E54" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F54" s="29">
@@ -2845,7 +2845,7 @@
       <c r="C55" s="31" t="n"/>
       <c r="D55" s="31" t="n"/>
       <c r="E55" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F55" s="29">
@@ -2859,7 +2859,7 @@
       <c r="C56" s="31" t="n"/>
       <c r="D56" s="31" t="n"/>
       <c r="E56" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F56" s="29">
@@ -2873,7 +2873,7 @@
       <c r="C57" s="31" t="n"/>
       <c r="D57" s="31" t="n"/>
       <c r="E57" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F57" s="29">
@@ -2887,7 +2887,7 @@
       <c r="C58" s="31" t="n"/>
       <c r="D58" s="31" t="n"/>
       <c r="E58" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F58" s="29">
@@ -2901,7 +2901,7 @@
       <c r="C59" s="31" t="n"/>
       <c r="D59" s="31" t="n"/>
       <c r="E59" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F59" s="29">
@@ -2915,7 +2915,7 @@
       <c r="C60" s="31" t="n"/>
       <c r="D60" s="31" t="n"/>
       <c r="E60" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F60" s="29">
@@ -2929,7 +2929,7 @@
       <c r="C61" s="31" t="n"/>
       <c r="D61" s="31" t="n"/>
       <c r="E61" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F61" s="29">
@@ -2943,7 +2943,7 @@
       <c r="C62" s="31" t="n"/>
       <c r="D62" s="31" t="n"/>
       <c r="E62" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F62" s="29">
@@ -2957,7 +2957,7 @@
       <c r="C63" s="31" t="n"/>
       <c r="D63" s="31" t="n"/>
       <c r="E63" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F63" s="29">
@@ -2971,7 +2971,7 @@
       <c r="C64" s="31" t="n"/>
       <c r="D64" s="31" t="n"/>
       <c r="E64" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F64" s="29">
@@ -2985,7 +2985,7 @@
       <c r="C65" s="31" t="n"/>
       <c r="D65" s="31" t="n"/>
       <c r="E65" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F65" s="29">
@@ -2999,7 +2999,7 @@
       <c r="C66" s="31" t="n"/>
       <c r="D66" s="31" t="n"/>
       <c r="E66" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F66" s="29">
@@ -3013,7 +3013,7 @@
       <c r="C67" s="31" t="n"/>
       <c r="D67" s="31" t="n"/>
       <c r="E67" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F67" s="29">
@@ -3027,7 +3027,7 @@
       <c r="C68" s="31" t="n"/>
       <c r="D68" s="31" t="n"/>
       <c r="E68" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F68" s="29">
@@ -3041,7 +3041,7 @@
       <c r="C69" s="31" t="n"/>
       <c r="D69" s="31" t="n"/>
       <c r="E69" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F69" s="29">
@@ -3055,7 +3055,7 @@
       <c r="C70" s="31" t="n"/>
       <c r="D70" s="31" t="n"/>
       <c r="E70" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F70" s="29">
@@ -3069,7 +3069,7 @@
       <c r="C71" s="31" t="n"/>
       <c r="D71" s="31" t="n"/>
       <c r="E71" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F71" s="29">
@@ -3083,7 +3083,7 @@
       <c r="C72" s="31" t="n"/>
       <c r="D72" s="31" t="n"/>
       <c r="E72" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F72" s="29">
@@ -3097,7 +3097,7 @@
       <c r="C73" s="31" t="n"/>
       <c r="D73" s="31" t="n"/>
       <c r="E73" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F73" s="29">
@@ -3111,7 +3111,7 @@
       <c r="C74" s="31" t="n"/>
       <c r="D74" s="31" t="n"/>
       <c r="E74" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F74" s="29">
@@ -3125,7 +3125,7 @@
       <c r="C75" s="31" t="n"/>
       <c r="D75" s="31" t="n"/>
       <c r="E75" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F75" s="29">
@@ -3139,7 +3139,7 @@
       <c r="C76" s="31" t="n"/>
       <c r="D76" s="31" t="n"/>
       <c r="E76" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F76" s="29">
@@ -3153,7 +3153,7 @@
       <c r="C77" s="31" t="n"/>
       <c r="D77" s="31" t="n"/>
       <c r="E77" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F77" s="29">
@@ -3167,7 +3167,7 @@
       <c r="C78" s="31" t="n"/>
       <c r="D78" s="31" t="n"/>
       <c r="E78" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F78" s="29">
@@ -3181,7 +3181,7 @@
       <c r="C79" s="31" t="n"/>
       <c r="D79" s="31" t="n"/>
       <c r="E79" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F79" s="29">
@@ -3195,7 +3195,7 @@
       <c r="C80" s="31" t="n"/>
       <c r="D80" s="31" t="n"/>
       <c r="E80" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F80" s="29">
@@ -3209,7 +3209,7 @@
       <c r="C81" s="31" t="n"/>
       <c r="D81" s="31" t="n"/>
       <c r="E81" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F81" s="29">
@@ -3223,7 +3223,7 @@
       <c r="C82" s="31" t="n"/>
       <c r="D82" s="31" t="n"/>
       <c r="E82" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F82" s="29">
@@ -3237,7 +3237,7 @@
       <c r="C83" s="31" t="n"/>
       <c r="D83" s="31" t="n"/>
       <c r="E83" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F83" s="29">
@@ -3251,7 +3251,7 @@
       <c r="C84" s="31" t="n"/>
       <c r="D84" s="31" t="n"/>
       <c r="E84" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F84" s="29">
@@ -3265,7 +3265,7 @@
       <c r="C85" s="31" t="n"/>
       <c r="D85" s="31" t="n"/>
       <c r="E85" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F85" s="29">
@@ -3279,7 +3279,7 @@
       <c r="C86" s="31" t="n"/>
       <c r="D86" s="31" t="n"/>
       <c r="E86" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F86" s="29">
@@ -3293,7 +3293,7 @@
       <c r="C87" s="31" t="n"/>
       <c r="D87" s="31" t="n"/>
       <c r="E87" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F87" s="29">
@@ -3307,7 +3307,7 @@
       <c r="C88" s="31" t="n"/>
       <c r="D88" s="31" t="n"/>
       <c r="E88" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F88" s="29">
@@ -3321,7 +3321,7 @@
       <c r="C89" s="31" t="n"/>
       <c r="D89" s="31" t="n"/>
       <c r="E89" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F89" s="29">
@@ -3335,7 +3335,7 @@
       <c r="C90" s="31" t="n"/>
       <c r="D90" s="31" t="n"/>
       <c r="E90" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F90" s="29">
@@ -3349,7 +3349,7 @@
       <c r="C91" s="31" t="n"/>
       <c r="D91" s="31" t="n"/>
       <c r="E91" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F91" s="29">
@@ -3363,7 +3363,7 @@
       <c r="C92" s="31" t="n"/>
       <c r="D92" s="31" t="n"/>
       <c r="E92" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F92" s="29">
@@ -3377,7 +3377,7 @@
       <c r="C93" s="31" t="n"/>
       <c r="D93" s="31" t="n"/>
       <c r="E93" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F93" s="29">
@@ -3391,7 +3391,7 @@
       <c r="C94" s="31" t="n"/>
       <c r="D94" s="31" t="n"/>
       <c r="E94" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F94" s="29">
@@ -3405,7 +3405,7 @@
       <c r="C95" s="31" t="n"/>
       <c r="D95" s="31" t="n"/>
       <c r="E95" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F95" s="29">
@@ -3419,7 +3419,7 @@
       <c r="C96" s="31" t="n"/>
       <c r="D96" s="31" t="n"/>
       <c r="E96" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F96" s="29">
@@ -3433,7 +3433,7 @@
       <c r="C97" s="31" t="n"/>
       <c r="D97" s="31" t="n"/>
       <c r="E97" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F97" s="29">
@@ -3447,7 +3447,7 @@
       <c r="C98" s="31" t="n"/>
       <c r="D98" s="31" t="n"/>
       <c r="E98" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F98" s="29">
@@ -3461,7 +3461,7 @@
       <c r="C99" s="31" t="n"/>
       <c r="D99" s="31" t="n"/>
       <c r="E99" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F99" s="29">
@@ -3475,7 +3475,7 @@
       <c r="C100" s="31" t="n"/>
       <c r="D100" s="31" t="n"/>
       <c r="E100" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F100" s="29">
@@ -3489,7 +3489,7 @@
       <c r="C101" s="31" t="n"/>
       <c r="D101" s="31" t="n"/>
       <c r="E101" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F101" s="29">
@@ -3503,7 +3503,7 @@
       <c r="C102" s="31" t="n"/>
       <c r="D102" s="31" t="n"/>
       <c r="E102" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F102" s="29">
@@ -3517,7 +3517,7 @@
       <c r="C103" s="31" t="n"/>
       <c r="D103" s="31" t="n"/>
       <c r="E103" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F103" s="29">
@@ -3531,7 +3531,7 @@
       <c r="C104" s="31" t="n"/>
       <c r="D104" s="31" t="n"/>
       <c r="E104" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F104" s="29">
@@ -3545,7 +3545,7 @@
       <c r="C105" s="31" t="n"/>
       <c r="D105" s="31" t="n"/>
       <c r="E105" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F105" s="29">
@@ -3559,7 +3559,7 @@
       <c r="C106" s="31" t="n"/>
       <c r="D106" s="31" t="n"/>
       <c r="E106" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F106" s="29">
@@ -3573,7 +3573,7 @@
       <c r="C107" s="31" t="n"/>
       <c r="D107" s="31" t="n"/>
       <c r="E107" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F107" s="29">
@@ -3587,7 +3587,7 @@
       <c r="C108" s="31" t="n"/>
       <c r="D108" s="31" t="n"/>
       <c r="E108" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F108" s="29">
@@ -3601,7 +3601,7 @@
       <c r="C109" s="31" t="n"/>
       <c r="D109" s="31" t="n"/>
       <c r="E109" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F109" s="29">
@@ -3615,7 +3615,7 @@
       <c r="C110" s="31" t="n"/>
       <c r="D110" s="31" t="n"/>
       <c r="E110" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F110" s="29">
@@ -3629,7 +3629,7 @@
       <c r="C111" s="31" t="n"/>
       <c r="D111" s="31" t="n"/>
       <c r="E111" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F111" s="29">
@@ -3643,7 +3643,7 @@
       <c r="C112" s="31" t="n"/>
       <c r="D112" s="31" t="n"/>
       <c r="E112" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F112" s="29">
@@ -3657,7 +3657,7 @@
       <c r="C113" s="31" t="n"/>
       <c r="D113" s="31" t="n"/>
       <c r="E113" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F113" s="29">
@@ -3671,7 +3671,7 @@
       <c r="C114" s="31" t="n"/>
       <c r="D114" s="31" t="n"/>
       <c r="E114" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F114" s="29">
@@ -3685,7 +3685,7 @@
       <c r="C115" s="31" t="n"/>
       <c r="D115" s="31" t="n"/>
       <c r="E115" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F115" s="29">
@@ -3699,7 +3699,7 @@
       <c r="C116" s="31" t="n"/>
       <c r="D116" s="31" t="n"/>
       <c r="E116" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F116" s="29">
@@ -3713,7 +3713,7 @@
       <c r="C117" s="31" t="n"/>
       <c r="D117" s="31" t="n"/>
       <c r="E117" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F117" s="29">
@@ -3727,7 +3727,7 @@
       <c r="C118" s="31" t="n"/>
       <c r="D118" s="31" t="n"/>
       <c r="E118" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F118" s="29">
@@ -3741,7 +3741,7 @@
       <c r="C119" s="31" t="n"/>
       <c r="D119" s="31" t="n"/>
       <c r="E119" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F119" s="29">
@@ -3755,7 +3755,7 @@
       <c r="C120" s="31" t="n"/>
       <c r="D120" s="31" t="n"/>
       <c r="E120" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F120" s="29">
@@ -3769,7 +3769,7 @@
       <c r="C121" s="31" t="n"/>
       <c r="D121" s="31" t="n"/>
       <c r="E121" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F121" s="29">
@@ -3783,7 +3783,7 @@
       <c r="C122" s="31" t="n"/>
       <c r="D122" s="31" t="n"/>
       <c r="E122" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F122" s="29">
@@ -3797,7 +3797,7 @@
       <c r="C123" s="31" t="n"/>
       <c r="D123" s="31" t="n"/>
       <c r="E123" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F123" s="29">
@@ -3811,7 +3811,7 @@
       <c r="C124" s="31" t="n"/>
       <c r="D124" s="31" t="n"/>
       <c r="E124" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F124" s="29">
@@ -3825,7 +3825,7 @@
       <c r="C125" s="31" t="n"/>
       <c r="D125" s="31" t="n"/>
       <c r="E125" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F125" s="29">
@@ -3839,7 +3839,7 @@
       <c r="C126" s="31" t="n"/>
       <c r="D126" s="31" t="n"/>
       <c r="E126" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F126" s="29">
@@ -3853,7 +3853,7 @@
       <c r="C127" s="31" t="n"/>
       <c r="D127" s="31" t="n"/>
       <c r="E127" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F127" s="29">
@@ -3867,7 +3867,7 @@
       <c r="C128" s="31" t="n"/>
       <c r="D128" s="31" t="n"/>
       <c r="E128" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F128" s="29">
@@ -3881,7 +3881,7 @@
       <c r="C129" s="31" t="n"/>
       <c r="D129" s="31" t="n"/>
       <c r="E129" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F129" s="29">
@@ -3895,7 +3895,7 @@
       <c r="C130" s="31" t="n"/>
       <c r="D130" s="31" t="n"/>
       <c r="E130" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F130" s="29">
@@ -3909,7 +3909,7 @@
       <c r="C131" s="31" t="n"/>
       <c r="D131" s="31" t="n"/>
       <c r="E131" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F131" s="29">
@@ -3923,7 +3923,7 @@
       <c r="C132" s="31" t="n"/>
       <c r="D132" s="31" t="n"/>
       <c r="E132" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F132" s="29">
@@ -3937,7 +3937,7 @@
       <c r="C133" s="31" t="n"/>
       <c r="D133" s="31" t="n"/>
       <c r="E133" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F133" s="29">
@@ -3951,7 +3951,7 @@
       <c r="C134" s="31" t="n"/>
       <c r="D134" s="31" t="n"/>
       <c r="E134" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F134" s="29">
@@ -3965,7 +3965,7 @@
       <c r="C135" s="31" t="n"/>
       <c r="D135" s="31" t="n"/>
       <c r="E135" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F135" s="29">
@@ -3979,7 +3979,7 @@
       <c r="C136" s="31" t="n"/>
       <c r="D136" s="31" t="n"/>
       <c r="E136" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F136" s="29">
@@ -3993,7 +3993,7 @@
       <c r="C137" s="31" t="n"/>
       <c r="D137" s="31" t="n"/>
       <c r="E137" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F137" s="29">
@@ -4007,7 +4007,7 @@
       <c r="C138" s="31" t="n"/>
       <c r="D138" s="31" t="n"/>
       <c r="E138" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F138" s="29">
@@ -4021,7 +4021,7 @@
       <c r="C139" s="31" t="n"/>
       <c r="D139" s="31" t="n"/>
       <c r="E139" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F139" s="29">
@@ -4035,7 +4035,7 @@
       <c r="C140" s="31" t="n"/>
       <c r="D140" s="31" t="n"/>
       <c r="E140" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F140" s="29">
@@ -4049,7 +4049,7 @@
       <c r="C141" s="31" t="n"/>
       <c r="D141" s="31" t="n"/>
       <c r="E141" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F141" s="29">
@@ -4063,7 +4063,7 @@
       <c r="C142" s="31" t="n"/>
       <c r="D142" s="31" t="n"/>
       <c r="E142" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F142" s="29">
@@ -4077,7 +4077,7 @@
       <c r="C143" s="31" t="n"/>
       <c r="D143" s="31" t="n"/>
       <c r="E143" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F143" s="29">
@@ -4091,7 +4091,7 @@
       <c r="C144" s="31" t="n"/>
       <c r="D144" s="31" t="n"/>
       <c r="E144" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F144" s="29">
@@ -4105,7 +4105,7 @@
       <c r="C145" s="31" t="n"/>
       <c r="D145" s="31" t="n"/>
       <c r="E145" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F145" s="29">
@@ -4119,7 +4119,7 @@
       <c r="C146" s="31" t="n"/>
       <c r="D146" s="31" t="n"/>
       <c r="E146" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F146" s="29">
@@ -4133,7 +4133,7 @@
       <c r="C147" s="31" t="n"/>
       <c r="D147" s="31" t="n"/>
       <c r="E147" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F147" s="29">
@@ -4147,7 +4147,7 @@
       <c r="C148" s="31" t="n"/>
       <c r="D148" s="31" t="n"/>
       <c r="E148" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F148" s="29">
@@ -4161,7 +4161,7 @@
       <c r="C149" s="31" t="n"/>
       <c r="D149" s="31" t="n"/>
       <c r="E149" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F149" s="29">
@@ -4175,7 +4175,7 @@
       <c r="C150" s="31" t="n"/>
       <c r="D150" s="31" t="n"/>
       <c r="E150" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F150" s="29">
@@ -4189,7 +4189,7 @@
       <c r="C151" s="31" t="n"/>
       <c r="D151" s="31" t="n"/>
       <c r="E151" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F151" s="29">
@@ -4203,7 +4203,7 @@
       <c r="C152" s="31" t="n"/>
       <c r="D152" s="31" t="n"/>
       <c r="E152" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F152" s="29">
@@ -4217,7 +4217,7 @@
       <c r="C153" s="31" t="n"/>
       <c r="D153" s="31" t="n"/>
       <c r="E153" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F153" s="29">
@@ -4231,7 +4231,7 @@
       <c r="C154" s="31" t="n"/>
       <c r="D154" s="31" t="n"/>
       <c r="E154" s="31">
-        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$DZ$300,TRIM(tblStock[[#This Row],[Item code]])))</f>
+        <f>IF(TRIM(tblStock[[#This Row],[Item code]])="","",COUNTIF(Map!$A$6:$ZZ$2000,TRIM(tblStock[[#This Row],[Item code]])))</f>
         <v/>
       </c>
       <c r="F154" s="29">

</xml_diff>